<commit_message>
Integracion completa de Categorias y RBAC (Limpieza de archivos pesados)
</commit_message>
<xml_diff>
--- a/backend/Template_archivo_plano/template_plano - copia.xlsx
+++ b/backend/Template_archivo_plano/template_plano - copia.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alejandro.carvajal\Documents\langextract_ocr\backend\Template_archivo_plano\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D09A13C4-2329-42D1-B3EE-605E6691FF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE4584A-FD8A-41BA-A093-BAC8A7FAE683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -172,7 +172,7 @@
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -195,12 +195,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -309,17 +303,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="8" applyFill="1"/>
@@ -329,12 +323,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="8" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Millares [0] 2" xfId="4" xr:uid="{73AE917C-989C-45DF-A9A9-58CBEAA1EF06}"/>
@@ -796,184 +789,184 @@
     </row>
     <row r="2" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D2" s="1"/>
-      <c r="E2" s="13"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="16"/>
-      <c r="L2" s="16"/>
-      <c r="M2" s="16"/>
+      <c r="E2" s="12"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
       <c r="AA2" s="2"/>
       <c r="AG2" s="10"/>
       <c r="AH2" s="11"/>
-      <c r="AK2" s="17"/>
+      <c r="AK2" s="16"/>
     </row>
     <row r="3" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D3" s="1"/>
-      <c r="E3" s="13"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
+      <c r="E3" s="12"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
       <c r="AA3" s="2"/>
       <c r="AG3" s="10"/>
       <c r="AH3" s="11"/>
-      <c r="AK3" s="17"/>
+      <c r="AK3" s="16"/>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D4" s="1"/>
-      <c r="E4" s="13"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
+      <c r="E4" s="12"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
       <c r="AA4" s="2"/>
       <c r="AG4" s="10"/>
       <c r="AH4" s="11"/>
-      <c r="AK4" s="17"/>
+      <c r="AK4" s="16"/>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D5" s="1"/>
-      <c r="E5" s="13"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="16"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="16"/>
+      <c r="E5" s="12"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
       <c r="AA5" s="2"/>
       <c r="AG5" s="10"/>
       <c r="AH5" s="11"/>
-      <c r="AK5" s="17"/>
+      <c r="AK5" s="16"/>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D6" s="1"/>
-      <c r="E6" s="13"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="16"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="16"/>
+      <c r="E6" s="12"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
       <c r="AA6" s="2"/>
       <c r="AG6" s="10"/>
       <c r="AH6" s="11"/>
-      <c r="AK6" s="17"/>
+      <c r="AK6" s="16"/>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D7" s="1"/>
-      <c r="E7" s="13"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
+      <c r="E7" s="12"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="15"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="15"/>
       <c r="AA7" s="2"/>
       <c r="AG7" s="10"/>
       <c r="AH7" s="11"/>
-      <c r="AK7" s="17"/>
+      <c r="AK7" s="16"/>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D8" s="1"/>
-      <c r="E8" s="13"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
+      <c r="E8" s="12"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
       <c r="AA8" s="2"/>
       <c r="AG8" s="10"/>
       <c r="AH8" s="11"/>
-      <c r="AK8" s="17"/>
+      <c r="AK8" s="16"/>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D9" s="1"/>
-      <c r="E9" s="13"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
+      <c r="E9" s="12"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="15"/>
       <c r="AA9" s="2"/>
       <c r="AG9" s="10"/>
       <c r="AH9" s="11"/>
-      <c r="AK9" s="17"/>
+      <c r="AK9" s="16"/>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D10" s="1"/>
-      <c r="E10" s="13"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
+      <c r="E10" s="12"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
       <c r="AA10" s="2"/>
       <c r="AG10" s="10"/>
       <c r="AH10" s="11"/>
-      <c r="AK10" s="17"/>
+      <c r="AK10" s="16"/>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D11" s="1"/>
-      <c r="E11" s="13"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
+      <c r="E11" s="12"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="15"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="15"/>
       <c r="AA11" s="2"/>
       <c r="AG11" s="10"/>
       <c r="AH11" s="11"/>
-      <c r="AK11" s="17"/>
+      <c r="AK11" s="16"/>
     </row>
     <row r="12" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D12" s="1"/>
-      <c r="E12" s="13"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
+      <c r="E12" s="12"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="14"/>
+      <c r="I12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
       <c r="AA12" s="2"/>
       <c r="AG12" s="10"/>
       <c r="AH12" s="11"/>
-      <c r="AK12" s="17"/>
+      <c r="AK12" s="16"/>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D13" s="1"/>
-      <c r="E13" s="13"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
+      <c r="E13" s="12"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="15"/>
+      <c r="L13" s="15"/>
+      <c r="M13" s="15"/>
       <c r="AA13" s="2"/>
       <c r="AG13" s="10"/>
       <c r="AH13" s="11"/>
-      <c r="AK13" s="17"/>
+      <c r="AK13" s="16"/>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D14" s="1"/>
-      <c r="E14" s="13"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
+      <c r="E14" s="12"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="15"/>
+      <c r="L14" s="15"/>
+      <c r="M14" s="15"/>
       <c r="AA14" s="2"/>
       <c r="AG14" s="10"/>
       <c r="AH14" s="11"/>
-      <c r="AK14" s="17"/>
+      <c r="AK14" s="16"/>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D15" s="1"/>
       <c r="G15" s="6"/>
       <c r="H15" s="7"/>
       <c r="I15" s="8"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
+      <c r="L15" s="15"/>
+      <c r="M15" s="15"/>
       <c r="AA15" s="2"/>
       <c r="AG15" s="10"/>
       <c r="AH15" s="11"/>
-      <c r="AK15" s="12"/>
+      <c r="AK15" s="16"/>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.35">
       <c r="D16" s="1"/>
@@ -981,11 +974,11 @@
       <c r="H16" s="7"/>
       <c r="I16" s="8"/>
       <c r="L16" s="6"/>
-      <c r="M16" s="16"/>
+      <c r="M16" s="15"/>
       <c r="AA16" s="2"/>
       <c r="AG16" s="10"/>
       <c r="AH16" s="11"/>
-      <c r="AK16" s="12"/>
+      <c r="AK16" s="16"/>
     </row>
     <row r="17" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D17" s="1"/>
@@ -993,11 +986,11 @@
       <c r="H17" s="7"/>
       <c r="I17" s="8"/>
       <c r="L17" s="6"/>
-      <c r="M17" s="16"/>
+      <c r="M17" s="15"/>
       <c r="AA17" s="2"/>
       <c r="AG17" s="10"/>
       <c r="AH17" s="11"/>
-      <c r="AK17" s="12"/>
+      <c r="AK17" s="16"/>
     </row>
     <row r="18" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D18" s="1"/>
@@ -1008,7 +1001,7 @@
       <c r="AA18" s="2"/>
       <c r="AG18" s="10"/>
       <c r="AH18" s="11"/>
-      <c r="AK18" s="12"/>
+      <c r="AK18" s="16"/>
     </row>
     <row r="19" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D19" s="1"/>
@@ -1019,7 +1012,7 @@
       <c r="AA19" s="2"/>
       <c r="AG19" s="10"/>
       <c r="AH19" s="11"/>
-      <c r="AK19" s="12"/>
+      <c r="AK19" s="16"/>
     </row>
     <row r="20" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D20" s="1"/>
@@ -1030,7 +1023,7 @@
       <c r="AA20" s="2"/>
       <c r="AG20" s="10"/>
       <c r="AH20" s="11"/>
-      <c r="AK20" s="12"/>
+      <c r="AK20" s="16"/>
     </row>
     <row r="21" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D21" s="1"/>
@@ -1041,7 +1034,7 @@
       <c r="AA21" s="2"/>
       <c r="AG21" s="10"/>
       <c r="AH21" s="11"/>
-      <c r="AK21" s="12"/>
+      <c r="AK21" s="16"/>
     </row>
     <row r="22" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D22" s="1"/>
@@ -1052,7 +1045,7 @@
       <c r="AA22" s="2"/>
       <c r="AG22" s="10"/>
       <c r="AH22" s="11"/>
-      <c r="AK22" s="12"/>
+      <c r="AK22" s="16"/>
     </row>
     <row r="23" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D23" s="1"/>
@@ -1063,7 +1056,7 @@
       <c r="AA23" s="2"/>
       <c r="AG23" s="10"/>
       <c r="AH23" s="11"/>
-      <c r="AK23" s="12"/>
+      <c r="AK23" s="16"/>
     </row>
     <row r="24" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D24" s="1"/>
@@ -1074,7 +1067,7 @@
       <c r="AA24" s="2"/>
       <c r="AG24" s="10"/>
       <c r="AH24" s="11"/>
-      <c r="AK24" s="12"/>
+      <c r="AK24" s="16"/>
     </row>
     <row r="25" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D25" s="1"/>
@@ -1085,7 +1078,7 @@
       <c r="AA25" s="2"/>
       <c r="AG25" s="10"/>
       <c r="AH25" s="11"/>
-      <c r="AK25" s="12"/>
+      <c r="AK25" s="16"/>
     </row>
     <row r="26" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D26" s="1"/>
@@ -1096,7 +1089,7 @@
       <c r="AA26" s="2"/>
       <c r="AG26" s="10"/>
       <c r="AH26" s="11"/>
-      <c r="AK26" s="12"/>
+      <c r="AK26" s="16"/>
     </row>
     <row r="27" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D27" s="1"/>
@@ -1107,7 +1100,7 @@
       <c r="AA27" s="2"/>
       <c r="AG27" s="10"/>
       <c r="AH27" s="11"/>
-      <c r="AK27" s="12"/>
+      <c r="AK27" s="16"/>
     </row>
     <row r="28" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D28" s="1"/>
@@ -1118,7 +1111,7 @@
       <c r="AA28" s="2"/>
       <c r="AG28" s="10"/>
       <c r="AH28" s="11"/>
-      <c r="AK28" s="12"/>
+      <c r="AK28" s="16"/>
     </row>
     <row r="29" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D29" s="1"/>
@@ -1129,7 +1122,7 @@
       <c r="AA29" s="2"/>
       <c r="AG29" s="10"/>
       <c r="AH29" s="11"/>
-      <c r="AK29" s="12"/>
+      <c r="AK29" s="16"/>
     </row>
     <row r="30" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D30" s="1"/>
@@ -1140,7 +1133,7 @@
       <c r="AA30" s="2"/>
       <c r="AG30" s="10"/>
       <c r="AH30" s="11"/>
-      <c r="AK30" s="12"/>
+      <c r="AK30" s="16"/>
     </row>
     <row r="31" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D31" s="1"/>
@@ -1151,7 +1144,7 @@
       <c r="AA31" s="2"/>
       <c r="AG31" s="10"/>
       <c r="AH31" s="11"/>
-      <c r="AK31" s="12"/>
+      <c r="AK31" s="16"/>
     </row>
     <row r="32" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D32" s="1"/>
@@ -1162,7 +1155,7 @@
       <c r="AA32" s="2"/>
       <c r="AG32" s="10"/>
       <c r="AH32" s="11"/>
-      <c r="AK32" s="12"/>
+      <c r="AK32" s="16"/>
     </row>
     <row r="33" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D33" s="1"/>
@@ -1173,7 +1166,7 @@
       <c r="AA33" s="2"/>
       <c r="AG33" s="10"/>
       <c r="AH33" s="11"/>
-      <c r="AK33" s="12"/>
+      <c r="AK33" s="16"/>
     </row>
     <row r="34" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D34" s="1"/>
@@ -1184,7 +1177,7 @@
       <c r="AA34" s="2"/>
       <c r="AG34" s="10"/>
       <c r="AH34" s="11"/>
-      <c r="AK34" s="12"/>
+      <c r="AK34" s="16"/>
     </row>
     <row r="35" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D35" s="1"/>
@@ -1195,7 +1188,7 @@
       <c r="AA35" s="2"/>
       <c r="AG35" s="10"/>
       <c r="AH35" s="11"/>
-      <c r="AK35" s="12"/>
+      <c r="AK35" s="16"/>
     </row>
     <row r="36" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D36" s="1"/>
@@ -1206,7 +1199,7 @@
       <c r="AA36" s="2"/>
       <c r="AG36" s="10"/>
       <c r="AH36" s="11"/>
-      <c r="AK36" s="12"/>
+      <c r="AK36" s="16"/>
     </row>
     <row r="37" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D37" s="1"/>
@@ -1217,7 +1210,7 @@
       <c r="AA37" s="2"/>
       <c r="AG37" s="10"/>
       <c r="AH37" s="11"/>
-      <c r="AK37" s="12"/>
+      <c r="AK37" s="16"/>
     </row>
     <row r="38" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D38" s="1"/>
@@ -1228,7 +1221,7 @@
       <c r="AA38" s="2"/>
       <c r="AG38" s="10"/>
       <c r="AH38" s="11"/>
-      <c r="AK38" s="12"/>
+      <c r="AK38" s="16"/>
     </row>
     <row r="39" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D39" s="1"/>
@@ -1239,7 +1232,7 @@
       <c r="AA39" s="2"/>
       <c r="AG39" s="10"/>
       <c r="AH39" s="11"/>
-      <c r="AK39" s="12"/>
+      <c r="AK39" s="16"/>
     </row>
     <row r="40" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D40" s="1"/>
@@ -1250,7 +1243,7 @@
       <c r="AA40" s="2"/>
       <c r="AG40" s="10"/>
       <c r="AH40" s="11"/>
-      <c r="AK40" s="12"/>
+      <c r="AK40" s="16"/>
     </row>
     <row r="41" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D41" s="1"/>
@@ -1261,7 +1254,7 @@
       <c r="AA41" s="2"/>
       <c r="AG41" s="10"/>
       <c r="AH41" s="11"/>
-      <c r="AK41" s="12"/>
+      <c r="AK41" s="16"/>
     </row>
     <row r="42" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D42" s="1"/>
@@ -1272,7 +1265,7 @@
       <c r="AA42" s="2"/>
       <c r="AG42" s="10"/>
       <c r="AH42" s="11"/>
-      <c r="AK42" s="12"/>
+      <c r="AK42" s="16"/>
     </row>
     <row r="43" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D43" s="1"/>
@@ -1283,7 +1276,7 @@
       <c r="AA43" s="2"/>
       <c r="AG43" s="10"/>
       <c r="AH43" s="11"/>
-      <c r="AK43" s="12"/>
+      <c r="AK43" s="16"/>
     </row>
     <row r="44" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D44" s="1"/>
@@ -1294,7 +1287,7 @@
       <c r="AA44" s="2"/>
       <c r="AG44" s="10"/>
       <c r="AH44" s="11"/>
-      <c r="AK44" s="12"/>
+      <c r="AK44" s="16"/>
     </row>
     <row r="45" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D45" s="1"/>
@@ -1305,7 +1298,7 @@
       <c r="AA45" s="2"/>
       <c r="AG45" s="10"/>
       <c r="AH45" s="11"/>
-      <c r="AK45" s="12"/>
+      <c r="AK45" s="16"/>
     </row>
     <row r="46" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D46" s="1"/>
@@ -1316,7 +1309,7 @@
       <c r="AA46" s="2"/>
       <c r="AG46" s="10"/>
       <c r="AH46" s="11"/>
-      <c r="AK46" s="12"/>
+      <c r="AK46" s="16"/>
     </row>
     <row r="47" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D47" s="1"/>
@@ -1327,7 +1320,7 @@
       <c r="AA47" s="2"/>
       <c r="AG47" s="10"/>
       <c r="AH47" s="11"/>
-      <c r="AK47" s="12"/>
+      <c r="AK47" s="16"/>
     </row>
     <row r="48" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D48" s="1"/>
@@ -1338,7 +1331,7 @@
       <c r="AA48" s="2"/>
       <c r="AG48" s="10"/>
       <c r="AH48" s="11"/>
-      <c r="AK48" s="12"/>
+      <c r="AK48" s="16"/>
     </row>
     <row r="49" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D49" s="1"/>
@@ -1349,7 +1342,7 @@
       <c r="AA49" s="2"/>
       <c r="AG49" s="10"/>
       <c r="AH49" s="11"/>
-      <c r="AK49" s="12"/>
+      <c r="AK49" s="16"/>
     </row>
     <row r="50" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D50" s="1"/>
@@ -1360,7 +1353,7 @@
       <c r="AA50" s="2"/>
       <c r="AG50" s="10"/>
       <c r="AH50" s="11"/>
-      <c r="AK50" s="12"/>
+      <c r="AK50" s="16"/>
     </row>
     <row r="51" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D51" s="1"/>
@@ -1371,7 +1364,7 @@
       <c r="AA51" s="2"/>
       <c r="AG51" s="10"/>
       <c r="AH51" s="11"/>
-      <c r="AK51" s="12"/>
+      <c r="AK51" s="16"/>
     </row>
     <row r="52" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D52" s="1"/>
@@ -1382,7 +1375,7 @@
       <c r="AA52" s="2"/>
       <c r="AG52" s="10"/>
       <c r="AH52" s="11"/>
-      <c r="AK52" s="12"/>
+      <c r="AK52" s="16"/>
     </row>
     <row r="53" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D53" s="1"/>
@@ -1393,7 +1386,7 @@
       <c r="AA53" s="2"/>
       <c r="AG53" s="10"/>
       <c r="AH53" s="11"/>
-      <c r="AK53" s="12"/>
+      <c r="AK53" s="16"/>
     </row>
     <row r="54" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D54" s="1"/>
@@ -1404,7 +1397,7 @@
       <c r="AA54" s="2"/>
       <c r="AG54" s="10"/>
       <c r="AH54" s="11"/>
-      <c r="AK54" s="12"/>
+      <c r="AK54" s="16"/>
     </row>
     <row r="55" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D55" s="1"/>
@@ -1415,7 +1408,7 @@
       <c r="AA55" s="2"/>
       <c r="AG55" s="10"/>
       <c r="AH55" s="11"/>
-      <c r="AK55" s="12"/>
+      <c r="AK55" s="16"/>
     </row>
     <row r="56" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D56" s="1"/>
@@ -1426,7 +1419,7 @@
       <c r="AA56" s="2"/>
       <c r="AG56" s="10"/>
       <c r="AH56" s="11"/>
-      <c r="AK56" s="12"/>
+      <c r="AK56" s="16"/>
     </row>
     <row r="57" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D57" s="1"/>
@@ -1437,7 +1430,7 @@
       <c r="AA57" s="2"/>
       <c r="AG57" s="10"/>
       <c r="AH57" s="11"/>
-      <c r="AK57" s="12"/>
+      <c r="AK57" s="16"/>
     </row>
     <row r="58" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D58" s="1"/>
@@ -1448,7 +1441,7 @@
       <c r="AA58" s="2"/>
       <c r="AG58" s="10"/>
       <c r="AH58" s="11"/>
-      <c r="AK58" s="12"/>
+      <c r="AK58" s="16"/>
     </row>
     <row r="59" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D59" s="1"/>
@@ -1459,7 +1452,7 @@
       <c r="AA59" s="2"/>
       <c r="AG59" s="10"/>
       <c r="AH59" s="11"/>
-      <c r="AK59" s="12"/>
+      <c r="AK59" s="16"/>
     </row>
     <row r="60" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D60" s="1"/>
@@ -1470,7 +1463,7 @@
       <c r="AA60" s="2"/>
       <c r="AG60" s="10"/>
       <c r="AH60" s="11"/>
-      <c r="AK60" s="12"/>
+      <c r="AK60" s="16"/>
     </row>
     <row r="61" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D61" s="1"/>
@@ -1481,7 +1474,7 @@
       <c r="AA61" s="2"/>
       <c r="AG61" s="10"/>
       <c r="AH61" s="11"/>
-      <c r="AK61" s="12"/>
+      <c r="AK61" s="16"/>
     </row>
     <row r="62" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D62" s="1"/>
@@ -1492,7 +1485,7 @@
       <c r="AA62" s="2"/>
       <c r="AG62" s="10"/>
       <c r="AH62" s="11"/>
-      <c r="AK62" s="12"/>
+      <c r="AK62" s="16"/>
     </row>
     <row r="63" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D63" s="1"/>
@@ -1503,7 +1496,7 @@
       <c r="AA63" s="2"/>
       <c r="AG63" s="10"/>
       <c r="AH63" s="11"/>
-      <c r="AK63" s="12"/>
+      <c r="AK63" s="16"/>
     </row>
     <row r="64" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D64" s="1"/>
@@ -1514,7 +1507,7 @@
       <c r="AA64" s="2"/>
       <c r="AG64" s="10"/>
       <c r="AH64" s="11"/>
-      <c r="AK64" s="12"/>
+      <c r="AK64" s="16"/>
     </row>
     <row r="65" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D65" s="1"/>
@@ -1525,7 +1518,7 @@
       <c r="AA65" s="2"/>
       <c r="AG65" s="10"/>
       <c r="AH65" s="11"/>
-      <c r="AK65" s="12"/>
+      <c r="AK65" s="16"/>
     </row>
     <row r="66" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D66" s="1"/>
@@ -1536,7 +1529,7 @@
       <c r="AA66" s="2"/>
       <c r="AG66" s="10"/>
       <c r="AH66" s="11"/>
-      <c r="AK66" s="12"/>
+      <c r="AK66" s="16"/>
     </row>
     <row r="67" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D67" s="1"/>
@@ -1547,7 +1540,7 @@
       <c r="AA67" s="2"/>
       <c r="AG67" s="10"/>
       <c r="AH67" s="11"/>
-      <c r="AK67" s="12"/>
+      <c r="AK67" s="16"/>
     </row>
     <row r="68" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D68" s="1"/>
@@ -1558,7 +1551,7 @@
       <c r="AA68" s="2"/>
       <c r="AG68" s="10"/>
       <c r="AH68" s="11"/>
-      <c r="AK68" s="12"/>
+      <c r="AK68" s="16"/>
     </row>
     <row r="69" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D69" s="1"/>
@@ -1569,7 +1562,7 @@
       <c r="AA69" s="2"/>
       <c r="AG69" s="10"/>
       <c r="AH69" s="11"/>
-      <c r="AK69" s="12"/>
+      <c r="AK69" s="16"/>
     </row>
     <row r="70" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D70" s="1"/>
@@ -1580,7 +1573,7 @@
       <c r="AA70" s="2"/>
       <c r="AG70" s="10"/>
       <c r="AH70" s="11"/>
-      <c r="AK70" s="12"/>
+      <c r="AK70" s="16"/>
     </row>
     <row r="71" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D71" s="1"/>
@@ -1591,7 +1584,7 @@
       <c r="AA71" s="2"/>
       <c r="AG71" s="10"/>
       <c r="AH71" s="11"/>
-      <c r="AK71" s="12"/>
+      <c r="AK71" s="16"/>
     </row>
     <row r="72" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D72" s="1"/>
@@ -1602,7 +1595,7 @@
       <c r="AA72" s="2"/>
       <c r="AG72" s="10"/>
       <c r="AH72" s="11"/>
-      <c r="AK72" s="12"/>
+      <c r="AK72" s="16"/>
     </row>
     <row r="73" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D73" s="1"/>
@@ -1613,7 +1606,7 @@
       <c r="AA73" s="2"/>
       <c r="AG73" s="10"/>
       <c r="AH73" s="11"/>
-      <c r="AK73" s="12"/>
+      <c r="AK73" s="16"/>
     </row>
     <row r="74" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D74" s="1"/>
@@ -1624,7 +1617,7 @@
       <c r="AA74" s="2"/>
       <c r="AG74" s="10"/>
       <c r="AH74" s="11"/>
-      <c r="AK74" s="12"/>
+      <c r="AK74" s="16"/>
     </row>
     <row r="75" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D75" s="1"/>
@@ -1635,7 +1628,7 @@
       <c r="AA75" s="2"/>
       <c r="AG75" s="10"/>
       <c r="AH75" s="11"/>
-      <c r="AK75" s="12"/>
+      <c r="AK75" s="16"/>
     </row>
     <row r="76" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D76" s="1"/>
@@ -1646,7 +1639,7 @@
       <c r="AA76" s="2"/>
       <c r="AG76" s="10"/>
       <c r="AH76" s="11"/>
-      <c r="AK76" s="12"/>
+      <c r="AK76" s="16"/>
     </row>
     <row r="77" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D77" s="1"/>
@@ -1657,7 +1650,7 @@
       <c r="AA77" s="2"/>
       <c r="AG77" s="10"/>
       <c r="AH77" s="11"/>
-      <c r="AK77" s="12"/>
+      <c r="AK77" s="16"/>
     </row>
     <row r="78" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D78" s="1"/>
@@ -1668,7 +1661,7 @@
       <c r="AA78" s="2"/>
       <c r="AG78" s="10"/>
       <c r="AH78" s="11"/>
-      <c r="AK78" s="12"/>
+      <c r="AK78" s="16"/>
     </row>
     <row r="79" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D79" s="1"/>
@@ -1679,7 +1672,7 @@
       <c r="AA79" s="2"/>
       <c r="AG79" s="10"/>
       <c r="AH79" s="11"/>
-      <c r="AK79" s="12"/>
+      <c r="AK79" s="16"/>
     </row>
     <row r="80" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D80" s="1"/>
@@ -1690,7 +1683,7 @@
       <c r="AA80" s="2"/>
       <c r="AG80" s="10"/>
       <c r="AH80" s="11"/>
-      <c r="AK80" s="12"/>
+      <c r="AK80" s="16"/>
     </row>
     <row r="81" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D81" s="1"/>
@@ -1701,7 +1694,7 @@
       <c r="AA81" s="2"/>
       <c r="AG81" s="10"/>
       <c r="AH81" s="11"/>
-      <c r="AK81" s="12"/>
+      <c r="AK81" s="16"/>
     </row>
     <row r="82" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D82" s="1"/>
@@ -1712,7 +1705,7 @@
       <c r="AA82" s="2"/>
       <c r="AG82" s="10"/>
       <c r="AH82" s="11"/>
-      <c r="AK82" s="12"/>
+      <c r="AK82" s="16"/>
     </row>
     <row r="83" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D83" s="1"/>
@@ -1723,7 +1716,7 @@
       <c r="AA83" s="2"/>
       <c r="AG83" s="10"/>
       <c r="AH83" s="11"/>
-      <c r="AK83" s="12"/>
+      <c r="AK83" s="16"/>
     </row>
     <row r="84" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D84" s="1"/>
@@ -1734,7 +1727,7 @@
       <c r="AA84" s="2"/>
       <c r="AG84" s="10"/>
       <c r="AH84" s="11"/>
-      <c r="AK84" s="12"/>
+      <c r="AK84" s="16"/>
     </row>
     <row r="85" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D85" s="1"/>
@@ -1745,7 +1738,7 @@
       <c r="AA85" s="2"/>
       <c r="AG85" s="10"/>
       <c r="AH85" s="11"/>
-      <c r="AK85" s="12"/>
+      <c r="AK85" s="16"/>
     </row>
     <row r="86" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D86" s="1"/>
@@ -1756,7 +1749,7 @@
       <c r="AA86" s="2"/>
       <c r="AG86" s="10"/>
       <c r="AH86" s="11"/>
-      <c r="AK86" s="12"/>
+      <c r="AK86" s="16"/>
     </row>
     <row r="87" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D87" s="1"/>
@@ -1767,7 +1760,7 @@
       <c r="AA87" s="2"/>
       <c r="AG87" s="10"/>
       <c r="AH87" s="11"/>
-      <c r="AK87" s="12"/>
+      <c r="AK87" s="16"/>
     </row>
     <row r="88" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D88" s="1"/>
@@ -1778,7 +1771,7 @@
       <c r="AA88" s="2"/>
       <c r="AG88" s="10"/>
       <c r="AH88" s="11"/>
-      <c r="AK88" s="12"/>
+      <c r="AK88" s="16"/>
     </row>
     <row r="89" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D89" s="1"/>
@@ -1789,7 +1782,7 @@
       <c r="AA89" s="2"/>
       <c r="AG89" s="10"/>
       <c r="AH89" s="11"/>
-      <c r="AK89" s="12"/>
+      <c r="AK89" s="16"/>
     </row>
     <row r="90" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D90" s="1"/>
@@ -1800,7 +1793,7 @@
       <c r="AA90" s="2"/>
       <c r="AG90" s="10"/>
       <c r="AH90" s="11"/>
-      <c r="AK90" s="12"/>
+      <c r="AK90" s="16"/>
     </row>
     <row r="91" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D91" s="1"/>
@@ -1811,7 +1804,7 @@
       <c r="AA91" s="2"/>
       <c r="AG91" s="10"/>
       <c r="AH91" s="11"/>
-      <c r="AK91" s="12"/>
+      <c r="AK91" s="16"/>
     </row>
     <row r="92" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D92" s="1"/>
@@ -1822,7 +1815,7 @@
       <c r="AA92" s="2"/>
       <c r="AG92" s="10"/>
       <c r="AH92" s="11"/>
-      <c r="AK92" s="12"/>
+      <c r="AK92" s="16"/>
     </row>
     <row r="93" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D93" s="1"/>
@@ -1833,7 +1826,7 @@
       <c r="AA93" s="2"/>
       <c r="AG93" s="10"/>
       <c r="AH93" s="11"/>
-      <c r="AK93" s="12"/>
+      <c r="AK93" s="16"/>
     </row>
     <row r="94" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D94" s="1"/>
@@ -1844,7 +1837,7 @@
       <c r="AA94" s="2"/>
       <c r="AG94" s="10"/>
       <c r="AH94" s="11"/>
-      <c r="AK94" s="12"/>
+      <c r="AK94" s="16"/>
     </row>
     <row r="95" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D95" s="1"/>
@@ -1855,7 +1848,7 @@
       <c r="AA95" s="2"/>
       <c r="AG95" s="10"/>
       <c r="AH95" s="11"/>
-      <c r="AK95" s="12"/>
+      <c r="AK95" s="16"/>
     </row>
     <row r="96" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D96" s="1"/>
@@ -1866,7 +1859,7 @@
       <c r="AA96" s="2"/>
       <c r="AG96" s="10"/>
       <c r="AH96" s="11"/>
-      <c r="AK96" s="12"/>
+      <c r="AK96" s="16"/>
     </row>
     <row r="97" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D97" s="1"/>
@@ -1877,7 +1870,7 @@
       <c r="AA97" s="2"/>
       <c r="AG97" s="10"/>
       <c r="AH97" s="11"/>
-      <c r="AK97" s="12"/>
+      <c r="AK97" s="16"/>
     </row>
     <row r="98" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D98" s="1"/>
@@ -1888,7 +1881,7 @@
       <c r="AA98" s="2"/>
       <c r="AG98" s="10"/>
       <c r="AH98" s="11"/>
-      <c r="AK98" s="12"/>
+      <c r="AK98" s="16"/>
     </row>
     <row r="99" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D99" s="1"/>
@@ -1899,7 +1892,7 @@
       <c r="AA99" s="2"/>
       <c r="AG99" s="10"/>
       <c r="AH99" s="11"/>
-      <c r="AK99" s="12"/>
+      <c r="AK99" s="16"/>
     </row>
     <row r="100" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D100" s="1"/>
@@ -1910,7 +1903,7 @@
       <c r="AA100" s="2"/>
       <c r="AG100" s="10"/>
       <c r="AH100" s="11"/>
-      <c r="AK100" s="12"/>
+      <c r="AK100" s="16"/>
     </row>
     <row r="101" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D101" s="1"/>
@@ -1921,7 +1914,7 @@
       <c r="AA101" s="2"/>
       <c r="AG101" s="10"/>
       <c r="AH101" s="11"/>
-      <c r="AK101" s="12"/>
+      <c r="AK101" s="16"/>
     </row>
     <row r="102" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D102" s="1"/>
@@ -1932,7 +1925,7 @@
       <c r="AA102" s="2"/>
       <c r="AG102" s="10"/>
       <c r="AH102" s="11"/>
-      <c r="AK102" s="12"/>
+      <c r="AK102" s="16"/>
     </row>
     <row r="103" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D103" s="1"/>
@@ -1943,7 +1936,7 @@
       <c r="AA103" s="2"/>
       <c r="AG103" s="10"/>
       <c r="AH103" s="11"/>
-      <c r="AK103" s="12"/>
+      <c r="AK103" s="16"/>
     </row>
     <row r="104" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D104" s="1"/>
@@ -1954,7 +1947,7 @@
       <c r="AA104" s="2"/>
       <c r="AG104" s="10"/>
       <c r="AH104" s="11"/>
-      <c r="AK104" s="12"/>
+      <c r="AK104" s="16"/>
     </row>
     <row r="105" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D105" s="1"/>
@@ -1965,7 +1958,7 @@
       <c r="AA105" s="2"/>
       <c r="AG105" s="10"/>
       <c r="AH105" s="11"/>
-      <c r="AK105" s="12"/>
+      <c r="AK105" s="16"/>
     </row>
     <row r="106" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D106" s="1"/>
@@ -1976,7 +1969,7 @@
       <c r="AA106" s="2"/>
       <c r="AG106" s="10"/>
       <c r="AH106" s="11"/>
-      <c r="AK106" s="12"/>
+      <c r="AK106" s="16"/>
     </row>
     <row r="107" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D107" s="1"/>
@@ -1987,7 +1980,7 @@
       <c r="AA107" s="2"/>
       <c r="AG107" s="10"/>
       <c r="AH107" s="11"/>
-      <c r="AK107" s="12"/>
+      <c r="AK107" s="16"/>
     </row>
     <row r="108" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D108" s="1"/>
@@ -1998,7 +1991,7 @@
       <c r="AA108" s="2"/>
       <c r="AG108" s="10"/>
       <c r="AH108" s="11"/>
-      <c r="AK108" s="12"/>
+      <c r="AK108" s="16"/>
     </row>
     <row r="109" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D109" s="1"/>
@@ -2009,7 +2002,7 @@
       <c r="AA109" s="2"/>
       <c r="AG109" s="10"/>
       <c r="AH109" s="11"/>
-      <c r="AK109" s="12"/>
+      <c r="AK109" s="16"/>
     </row>
     <row r="110" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D110" s="1"/>
@@ -2020,7 +2013,7 @@
       <c r="AA110" s="2"/>
       <c r="AG110" s="10"/>
       <c r="AH110" s="11"/>
-      <c r="AK110" s="12"/>
+      <c r="AK110" s="16"/>
     </row>
     <row r="111" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D111" s="1"/>
@@ -2031,7 +2024,7 @@
       <c r="AA111" s="2"/>
       <c r="AG111" s="10"/>
       <c r="AH111" s="11"/>
-      <c r="AK111" s="12"/>
+      <c r="AK111" s="16"/>
     </row>
     <row r="112" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D112" s="1"/>
@@ -2042,7 +2035,7 @@
       <c r="AA112" s="2"/>
       <c r="AG112" s="10"/>
       <c r="AH112" s="11"/>
-      <c r="AK112" s="12"/>
+      <c r="AK112" s="16"/>
     </row>
     <row r="113" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D113" s="1"/>
@@ -2053,7 +2046,7 @@
       <c r="AA113" s="2"/>
       <c r="AG113" s="10"/>
       <c r="AH113" s="11"/>
-      <c r="AK113" s="12"/>
+      <c r="AK113" s="16"/>
     </row>
     <row r="114" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D114" s="1"/>
@@ -2064,7 +2057,7 @@
       <c r="AA114" s="2"/>
       <c r="AG114" s="10"/>
       <c r="AH114" s="11"/>
-      <c r="AK114" s="12"/>
+      <c r="AK114" s="16"/>
     </row>
     <row r="115" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D115" s="1"/>
@@ -2075,7 +2068,7 @@
       <c r="AA115" s="2"/>
       <c r="AG115" s="10"/>
       <c r="AH115" s="11"/>
-      <c r="AK115" s="12"/>
+      <c r="AK115" s="16"/>
     </row>
     <row r="116" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D116" s="1"/>
@@ -2086,7 +2079,7 @@
       <c r="AA116" s="2"/>
       <c r="AG116" s="10"/>
       <c r="AH116" s="11"/>
-      <c r="AK116" s="12"/>
+      <c r="AK116" s="16"/>
     </row>
     <row r="117" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D117" s="1"/>
@@ -2097,7 +2090,7 @@
       <c r="AA117" s="2"/>
       <c r="AG117" s="10"/>
       <c r="AH117" s="11"/>
-      <c r="AK117" s="12"/>
+      <c r="AK117" s="16"/>
     </row>
     <row r="118" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D118" s="1"/>
@@ -2108,7 +2101,7 @@
       <c r="AA118" s="2"/>
       <c r="AG118" s="10"/>
       <c r="AH118" s="11"/>
-      <c r="AK118" s="12"/>
+      <c r="AK118" s="16"/>
     </row>
     <row r="119" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D119" s="1"/>
@@ -2119,7 +2112,7 @@
       <c r="AA119" s="2"/>
       <c r="AG119" s="10"/>
       <c r="AH119" s="11"/>
-      <c r="AK119" s="12"/>
+      <c r="AK119" s="16"/>
     </row>
     <row r="120" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D120" s="1"/>
@@ -2130,7 +2123,7 @@
       <c r="AA120" s="2"/>
       <c r="AG120" s="10"/>
       <c r="AH120" s="11"/>
-      <c r="AK120" s="12"/>
+      <c r="AK120" s="16"/>
     </row>
     <row r="121" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D121" s="1"/>
@@ -2141,7 +2134,7 @@
       <c r="AA121" s="2"/>
       <c r="AG121" s="10"/>
       <c r="AH121" s="11"/>
-      <c r="AK121" s="12"/>
+      <c r="AK121" s="16"/>
     </row>
     <row r="122" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D122" s="1"/>
@@ -2152,7 +2145,7 @@
       <c r="AA122" s="2"/>
       <c r="AG122" s="10"/>
       <c r="AH122" s="11"/>
-      <c r="AK122" s="12"/>
+      <c r="AK122" s="16"/>
     </row>
     <row r="123" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D123" s="1"/>
@@ -2163,7 +2156,7 @@
       <c r="AA123" s="2"/>
       <c r="AG123" s="10"/>
       <c r="AH123" s="11"/>
-      <c r="AK123" s="12"/>
+      <c r="AK123" s="16"/>
     </row>
     <row r="124" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D124" s="1"/>
@@ -2174,7 +2167,7 @@
       <c r="AA124" s="2"/>
       <c r="AG124" s="10"/>
       <c r="AH124" s="11"/>
-      <c r="AK124" s="12"/>
+      <c r="AK124" s="16"/>
     </row>
     <row r="125" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D125" s="1"/>
@@ -2185,7 +2178,7 @@
       <c r="AA125" s="2"/>
       <c r="AG125" s="10"/>
       <c r="AH125" s="11"/>
-      <c r="AK125" s="12"/>
+      <c r="AK125" s="16"/>
     </row>
     <row r="126" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D126" s="1"/>
@@ -2196,7 +2189,7 @@
       <c r="AA126" s="2"/>
       <c r="AG126" s="10"/>
       <c r="AH126" s="11"/>
-      <c r="AK126" s="12"/>
+      <c r="AK126" s="16"/>
     </row>
     <row r="127" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D127" s="1"/>
@@ -2207,7 +2200,7 @@
       <c r="AA127" s="2"/>
       <c r="AG127" s="10"/>
       <c r="AH127" s="11"/>
-      <c r="AK127" s="12"/>
+      <c r="AK127" s="16"/>
     </row>
     <row r="128" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D128" s="1"/>
@@ -2218,7 +2211,7 @@
       <c r="AA128" s="2"/>
       <c r="AG128" s="10"/>
       <c r="AH128" s="11"/>
-      <c r="AK128" s="12"/>
+      <c r="AK128" s="16"/>
     </row>
     <row r="129" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D129" s="1"/>
@@ -2229,7 +2222,7 @@
       <c r="AA129" s="2"/>
       <c r="AG129" s="10"/>
       <c r="AH129" s="11"/>
-      <c r="AK129" s="12"/>
+      <c r="AK129" s="16"/>
     </row>
     <row r="130" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D130" s="1"/>
@@ -2240,7 +2233,7 @@
       <c r="AA130" s="2"/>
       <c r="AG130" s="10"/>
       <c r="AH130" s="11"/>
-      <c r="AK130" s="12"/>
+      <c r="AK130" s="16"/>
     </row>
     <row r="131" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D131" s="1"/>
@@ -2251,7 +2244,7 @@
       <c r="AA131" s="2"/>
       <c r="AG131" s="10"/>
       <c r="AH131" s="11"/>
-      <c r="AK131" s="12"/>
+      <c r="AK131" s="16"/>
     </row>
     <row r="132" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D132" s="1"/>
@@ -2262,7 +2255,7 @@
       <c r="AA132" s="2"/>
       <c r="AG132" s="10"/>
       <c r="AH132" s="11"/>
-      <c r="AK132" s="12"/>
+      <c r="AK132" s="16"/>
     </row>
     <row r="133" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D133" s="1"/>
@@ -2273,7 +2266,7 @@
       <c r="AA133" s="2"/>
       <c r="AG133" s="10"/>
       <c r="AH133" s="11"/>
-      <c r="AK133" s="12"/>
+      <c r="AK133" s="16"/>
     </row>
     <row r="134" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D134" s="1"/>
@@ -2284,7 +2277,7 @@
       <c r="AA134" s="2"/>
       <c r="AG134" s="10"/>
       <c r="AH134" s="11"/>
-      <c r="AK134" s="12"/>
+      <c r="AK134" s="16"/>
     </row>
     <row r="135" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D135" s="1"/>
@@ -2295,7 +2288,7 @@
       <c r="AA135" s="2"/>
       <c r="AG135" s="10"/>
       <c r="AH135" s="11"/>
-      <c r="AK135" s="12"/>
+      <c r="AK135" s="16"/>
     </row>
     <row r="136" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D136" s="1"/>
@@ -2306,7 +2299,7 @@
       <c r="AA136" s="2"/>
       <c r="AG136" s="10"/>
       <c r="AH136" s="11"/>
-      <c r="AK136" s="12"/>
+      <c r="AK136" s="16"/>
     </row>
     <row r="137" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D137" s="1"/>
@@ -2317,7 +2310,7 @@
       <c r="AA137" s="2"/>
       <c r="AG137" s="10"/>
       <c r="AH137" s="11"/>
-      <c r="AK137" s="12"/>
+      <c r="AK137" s="16"/>
     </row>
     <row r="138" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D138" s="1"/>
@@ -2328,7 +2321,7 @@
       <c r="AA138" s="2"/>
       <c r="AG138" s="10"/>
       <c r="AH138" s="11"/>
-      <c r="AK138" s="12"/>
+      <c r="AK138" s="16"/>
     </row>
     <row r="139" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D139" s="1"/>
@@ -2339,7 +2332,7 @@
       <c r="AA139" s="2"/>
       <c r="AG139" s="10"/>
       <c r="AH139" s="11"/>
-      <c r="AK139" s="12"/>
+      <c r="AK139" s="16"/>
     </row>
     <row r="140" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D140" s="1"/>
@@ -2350,7 +2343,7 @@
       <c r="AA140" s="2"/>
       <c r="AG140" s="10"/>
       <c r="AH140" s="11"/>
-      <c r="AK140" s="12"/>
+      <c r="AK140" s="16"/>
     </row>
     <row r="141" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D141" s="1"/>
@@ -2361,7 +2354,7 @@
       <c r="AA141" s="2"/>
       <c r="AG141" s="10"/>
       <c r="AH141" s="11"/>
-      <c r="AK141" s="12"/>
+      <c r="AK141" s="16"/>
     </row>
     <row r="142" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D142" s="1"/>
@@ -2372,7 +2365,7 @@
       <c r="AA142" s="2"/>
       <c r="AG142" s="10"/>
       <c r="AH142" s="11"/>
-      <c r="AK142" s="12"/>
+      <c r="AK142" s="16"/>
     </row>
     <row r="143" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D143" s="1"/>
@@ -2383,7 +2376,7 @@
       <c r="AA143" s="2"/>
       <c r="AG143" s="10"/>
       <c r="AH143" s="11"/>
-      <c r="AK143" s="12"/>
+      <c r="AK143" s="16"/>
     </row>
     <row r="144" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D144" s="1"/>
@@ -2394,7 +2387,7 @@
       <c r="AA144" s="2"/>
       <c r="AG144" s="10"/>
       <c r="AH144" s="11"/>
-      <c r="AK144" s="12"/>
+      <c r="AK144" s="16"/>
     </row>
     <row r="145" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D145" s="1"/>
@@ -2405,7 +2398,7 @@
       <c r="AA145" s="2"/>
       <c r="AG145" s="10"/>
       <c r="AH145" s="11"/>
-      <c r="AK145" s="12"/>
+      <c r="AK145" s="16"/>
     </row>
     <row r="146" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D146" s="1"/>
@@ -2416,7 +2409,7 @@
       <c r="AA146" s="2"/>
       <c r="AG146" s="10"/>
       <c r="AH146" s="11"/>
-      <c r="AK146" s="12"/>
+      <c r="AK146" s="16"/>
     </row>
     <row r="147" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D147" s="1"/>
@@ -2427,7 +2420,7 @@
       <c r="AA147" s="2"/>
       <c r="AG147" s="10"/>
       <c r="AH147" s="11"/>
-      <c r="AK147" s="12"/>
+      <c r="AK147" s="16"/>
     </row>
     <row r="148" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D148" s="1"/>
@@ -2438,7 +2431,7 @@
       <c r="AA148" s="2"/>
       <c r="AG148" s="10"/>
       <c r="AH148" s="11"/>
-      <c r="AK148" s="12"/>
+      <c r="AK148" s="16"/>
     </row>
     <row r="149" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D149" s="1"/>
@@ -2449,7 +2442,7 @@
       <c r="AA149" s="2"/>
       <c r="AG149" s="10"/>
       <c r="AH149" s="11"/>
-      <c r="AK149" s="12"/>
+      <c r="AK149" s="16"/>
     </row>
     <row r="150" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D150" s="1"/>
@@ -2460,7 +2453,7 @@
       <c r="AA150" s="2"/>
       <c r="AG150" s="10"/>
       <c r="AH150" s="11"/>
-      <c r="AK150" s="12"/>
+      <c r="AK150" s="16"/>
     </row>
     <row r="151" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D151" s="1"/>
@@ -2471,7 +2464,7 @@
       <c r="AA151" s="2"/>
       <c r="AG151" s="10"/>
       <c r="AH151" s="11"/>
-      <c r="AK151" s="12"/>
+      <c r="AK151" s="16"/>
     </row>
     <row r="152" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D152" s="1"/>
@@ -2482,7 +2475,7 @@
       <c r="AA152" s="2"/>
       <c r="AG152" s="10"/>
       <c r="AH152" s="11"/>
-      <c r="AK152" s="12"/>
+      <c r="AK152" s="16"/>
     </row>
     <row r="153" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D153" s="1"/>
@@ -2493,7 +2486,7 @@
       <c r="AA153" s="2"/>
       <c r="AG153" s="10"/>
       <c r="AH153" s="11"/>
-      <c r="AK153" s="12"/>
+      <c r="AK153" s="16"/>
     </row>
     <row r="154" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D154" s="1"/>
@@ -2504,7 +2497,7 @@
       <c r="AA154" s="2"/>
       <c r="AG154" s="10"/>
       <c r="AH154" s="11"/>
-      <c r="AK154" s="12"/>
+      <c r="AK154" s="16"/>
     </row>
     <row r="155" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D155" s="1"/>
@@ -2515,7 +2508,7 @@
       <c r="AA155" s="2"/>
       <c r="AG155" s="10"/>
       <c r="AH155" s="11"/>
-      <c r="AK155" s="12"/>
+      <c r="AK155" s="16"/>
     </row>
     <row r="156" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D156" s="1"/>
@@ -2526,7 +2519,7 @@
       <c r="AA156" s="2"/>
       <c r="AG156" s="10"/>
       <c r="AH156" s="11"/>
-      <c r="AK156" s="12"/>
+      <c r="AK156" s="16"/>
     </row>
     <row r="157" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D157" s="1"/>
@@ -2537,7 +2530,7 @@
       <c r="AA157" s="2"/>
       <c r="AG157" s="10"/>
       <c r="AH157" s="11"/>
-      <c r="AK157" s="12"/>
+      <c r="AK157" s="16"/>
     </row>
     <row r="158" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D158" s="1"/>
@@ -2548,7 +2541,7 @@
       <c r="AA158" s="2"/>
       <c r="AG158" s="10"/>
       <c r="AH158" s="11"/>
-      <c r="AK158" s="12"/>
+      <c r="AK158" s="16"/>
     </row>
     <row r="159" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D159" s="1"/>
@@ -2559,7 +2552,7 @@
       <c r="AA159" s="2"/>
       <c r="AG159" s="10"/>
       <c r="AH159" s="11"/>
-      <c r="AK159" s="12"/>
+      <c r="AK159" s="16"/>
     </row>
     <row r="160" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D160" s="1"/>
@@ -2570,7 +2563,7 @@
       <c r="AA160" s="2"/>
       <c r="AG160" s="10"/>
       <c r="AH160" s="11"/>
-      <c r="AK160" s="12"/>
+      <c r="AK160" s="16"/>
     </row>
     <row r="161" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D161" s="1"/>
@@ -2581,7 +2574,7 @@
       <c r="AA161" s="2"/>
       <c r="AG161" s="10"/>
       <c r="AH161" s="11"/>
-      <c r="AK161" s="12"/>
+      <c r="AK161" s="16"/>
     </row>
     <row r="162" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D162" s="1"/>
@@ -2592,7 +2585,7 @@
       <c r="AA162" s="2"/>
       <c r="AG162" s="10"/>
       <c r="AH162" s="11"/>
-      <c r="AK162" s="12"/>
+      <c r="AK162" s="16"/>
     </row>
     <row r="163" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D163" s="1"/>
@@ -2603,7 +2596,7 @@
       <c r="AA163" s="2"/>
       <c r="AG163" s="10"/>
       <c r="AH163" s="11"/>
-      <c r="AK163" s="12"/>
+      <c r="AK163" s="16"/>
     </row>
     <row r="164" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D164" s="1"/>
@@ -2614,7 +2607,7 @@
       <c r="AA164" s="2"/>
       <c r="AG164" s="10"/>
       <c r="AH164" s="11"/>
-      <c r="AK164" s="12"/>
+      <c r="AK164" s="16"/>
     </row>
     <row r="165" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D165" s="1"/>
@@ -2625,7 +2618,7 @@
       <c r="AA165" s="2"/>
       <c r="AG165" s="10"/>
       <c r="AH165" s="11"/>
-      <c r="AK165" s="12"/>
+      <c r="AK165" s="16"/>
     </row>
     <row r="166" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D166" s="1"/>
@@ -2636,7 +2629,7 @@
       <c r="AA166" s="2"/>
       <c r="AG166" s="10"/>
       <c r="AH166" s="11"/>
-      <c r="AK166" s="12"/>
+      <c r="AK166" s="16"/>
     </row>
     <row r="167" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D167" s="1"/>
@@ -2647,7 +2640,7 @@
       <c r="AA167" s="2"/>
       <c r="AG167" s="10"/>
       <c r="AH167" s="11"/>
-      <c r="AK167" s="12"/>
+      <c r="AK167" s="16"/>
     </row>
     <row r="168" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D168" s="1"/>
@@ -2658,7 +2651,7 @@
       <c r="AA168" s="2"/>
       <c r="AG168" s="10"/>
       <c r="AH168" s="11"/>
-      <c r="AK168" s="12"/>
+      <c r="AK168" s="16"/>
     </row>
     <row r="169" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D169" s="1"/>
@@ -2669,7 +2662,7 @@
       <c r="AA169" s="2"/>
       <c r="AG169" s="10"/>
       <c r="AH169" s="11"/>
-      <c r="AK169" s="12"/>
+      <c r="AK169" s="16"/>
     </row>
     <row r="170" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D170" s="1"/>
@@ -2680,7 +2673,7 @@
       <c r="AA170" s="2"/>
       <c r="AG170" s="10"/>
       <c r="AH170" s="11"/>
-      <c r="AK170" s="12"/>
+      <c r="AK170" s="16"/>
     </row>
     <row r="171" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D171" s="1"/>
@@ -2691,7 +2684,7 @@
       <c r="AA171" s="2"/>
       <c r="AG171" s="10"/>
       <c r="AH171" s="11"/>
-      <c r="AK171" s="12"/>
+      <c r="AK171" s="16"/>
     </row>
     <row r="172" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D172" s="1"/>
@@ -2702,7 +2695,7 @@
       <c r="AA172" s="2"/>
       <c r="AG172" s="10"/>
       <c r="AH172" s="11"/>
-      <c r="AK172" s="12"/>
+      <c r="AK172" s="16"/>
     </row>
     <row r="173" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D173" s="1"/>
@@ -2713,7 +2706,7 @@
       <c r="AA173" s="2"/>
       <c r="AG173" s="10"/>
       <c r="AH173" s="11"/>
-      <c r="AK173" s="12"/>
+      <c r="AK173" s="16"/>
     </row>
     <row r="174" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D174" s="1"/>
@@ -2724,7 +2717,7 @@
       <c r="AA174" s="2"/>
       <c r="AG174" s="10"/>
       <c r="AH174" s="11"/>
-      <c r="AK174" s="12"/>
+      <c r="AK174" s="16"/>
     </row>
     <row r="175" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D175" s="1"/>
@@ -2735,7 +2728,7 @@
       <c r="AA175" s="2"/>
       <c r="AG175" s="10"/>
       <c r="AH175" s="11"/>
-      <c r="AK175" s="12"/>
+      <c r="AK175" s="16"/>
     </row>
     <row r="176" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D176" s="1"/>
@@ -2746,7 +2739,7 @@
       <c r="AA176" s="2"/>
       <c r="AG176" s="10"/>
       <c r="AH176" s="11"/>
-      <c r="AK176" s="12"/>
+      <c r="AK176" s="16"/>
     </row>
     <row r="177" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D177" s="1"/>
@@ -2757,7 +2750,7 @@
       <c r="AA177" s="2"/>
       <c r="AG177" s="10"/>
       <c r="AH177" s="11"/>
-      <c r="AK177" s="12"/>
+      <c r="AK177" s="16"/>
     </row>
     <row r="178" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D178" s="1"/>
@@ -2768,7 +2761,7 @@
       <c r="AA178" s="2"/>
       <c r="AG178" s="10"/>
       <c r="AH178" s="11"/>
-      <c r="AK178" s="12"/>
+      <c r="AK178" s="16"/>
     </row>
     <row r="179" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D179" s="1"/>
@@ -2779,7 +2772,7 @@
       <c r="AA179" s="2"/>
       <c r="AG179" s="10"/>
       <c r="AH179" s="11"/>
-      <c r="AK179" s="12"/>
+      <c r="AK179" s="16"/>
     </row>
     <row r="180" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D180" s="1"/>
@@ -2790,7 +2783,7 @@
       <c r="AA180" s="2"/>
       <c r="AG180" s="10"/>
       <c r="AH180" s="11"/>
-      <c r="AK180" s="12"/>
+      <c r="AK180" s="16"/>
     </row>
     <row r="181" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D181" s="1"/>
@@ -2801,7 +2794,7 @@
       <c r="AA181" s="2"/>
       <c r="AG181" s="11"/>
       <c r="AH181" s="10"/>
-      <c r="AK181" s="12"/>
+      <c r="AK181" s="16"/>
     </row>
     <row r="182" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D182" s="1"/>
@@ -2812,7 +2805,7 @@
       <c r="AA182" s="2"/>
       <c r="AG182" s="11"/>
       <c r="AH182" s="10"/>
-      <c r="AK182" s="12"/>
+      <c r="AK182" s="16"/>
     </row>
     <row r="183" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D183" s="1"/>
@@ -2823,7 +2816,7 @@
       <c r="AA183" s="2"/>
       <c r="AG183" s="11"/>
       <c r="AH183" s="10"/>
-      <c r="AK183" s="12"/>
+      <c r="AK183" s="16"/>
     </row>
     <row r="184" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D184" s="1"/>
@@ -2834,7 +2827,7 @@
       <c r="AA184" s="2"/>
       <c r="AG184" s="11"/>
       <c r="AH184" s="10"/>
-      <c r="AK184" s="12"/>
+      <c r="AK184" s="16"/>
     </row>
     <row r="185" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D185" s="1"/>
@@ -2845,7 +2838,7 @@
       <c r="AA185" s="2"/>
       <c r="AG185" s="11"/>
       <c r="AH185" s="10"/>
-      <c r="AK185" s="12"/>
+      <c r="AK185" s="16"/>
     </row>
     <row r="186" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D186" s="1"/>
@@ -2856,7 +2849,7 @@
       <c r="AA186" s="2"/>
       <c r="AG186" s="11"/>
       <c r="AH186" s="10"/>
-      <c r="AK186" s="12"/>
+      <c r="AK186" s="16"/>
     </row>
     <row r="187" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D187" s="1"/>
@@ -2867,7 +2860,7 @@
       <c r="AA187" s="2"/>
       <c r="AG187" s="11"/>
       <c r="AH187" s="10"/>
-      <c r="AK187" s="12"/>
+      <c r="AK187" s="16"/>
     </row>
     <row r="188" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D188" s="1"/>
@@ -2878,7 +2871,7 @@
       <c r="AA188" s="2"/>
       <c r="AG188" s="11"/>
       <c r="AH188" s="10"/>
-      <c r="AK188" s="12"/>
+      <c r="AK188" s="16"/>
     </row>
     <row r="189" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D189" s="1"/>
@@ -2889,7 +2882,7 @@
       <c r="AA189" s="2"/>
       <c r="AG189" s="11"/>
       <c r="AH189" s="10"/>
-      <c r="AK189" s="12"/>
+      <c r="AK189" s="16"/>
     </row>
     <row r="190" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D190" s="1"/>
@@ -2900,7 +2893,7 @@
       <c r="AA190" s="2"/>
       <c r="AG190" s="11"/>
       <c r="AH190" s="10"/>
-      <c r="AK190" s="12"/>
+      <c r="AK190" s="16"/>
     </row>
     <row r="191" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D191" s="1"/>
@@ -2911,7 +2904,7 @@
       <c r="AA191" s="2"/>
       <c r="AG191" s="11"/>
       <c r="AH191" s="10"/>
-      <c r="AK191" s="12"/>
+      <c r="AK191" s="16"/>
     </row>
     <row r="192" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D192" s="1"/>
@@ -2922,7 +2915,7 @@
       <c r="AA192" s="2"/>
       <c r="AG192" s="11"/>
       <c r="AH192" s="10"/>
-      <c r="AK192" s="12"/>
+      <c r="AK192" s="16"/>
     </row>
     <row r="193" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D193" s="1"/>
@@ -2933,7 +2926,7 @@
       <c r="AA193" s="2"/>
       <c r="AG193" s="11"/>
       <c r="AH193" s="10"/>
-      <c r="AK193" s="12"/>
+      <c r="AK193" s="16"/>
     </row>
     <row r="194" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D194" s="1"/>
@@ -2944,7 +2937,7 @@
       <c r="AA194" s="2"/>
       <c r="AG194" s="11"/>
       <c r="AH194" s="10"/>
-      <c r="AK194" s="12"/>
+      <c r="AK194" s="16"/>
     </row>
     <row r="195" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D195" s="1"/>
@@ -2955,7 +2948,7 @@
       <c r="AA195" s="2"/>
       <c r="AG195" s="11"/>
       <c r="AH195" s="10"/>
-      <c r="AK195" s="12"/>
+      <c r="AK195" s="16"/>
     </row>
     <row r="196" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D196" s="1"/>
@@ -2966,7 +2959,7 @@
       <c r="AA196" s="2"/>
       <c r="AG196" s="11"/>
       <c r="AH196" s="10"/>
-      <c r="AK196" s="12"/>
+      <c r="AK196" s="16"/>
     </row>
     <row r="197" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D197" s="1"/>
@@ -2977,7 +2970,7 @@
       <c r="AA197" s="2"/>
       <c r="AG197" s="11"/>
       <c r="AH197" s="10"/>
-      <c r="AK197" s="12"/>
+      <c r="AK197" s="16"/>
     </row>
     <row r="198" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D198" s="1"/>
@@ -2988,7 +2981,7 @@
       <c r="AA198" s="2"/>
       <c r="AG198" s="11"/>
       <c r="AH198" s="10"/>
-      <c r="AK198" s="12"/>
+      <c r="AK198" s="16"/>
     </row>
     <row r="199" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D199" s="1"/>
@@ -2999,7 +2992,7 @@
       <c r="AA199" s="2"/>
       <c r="AG199" s="11"/>
       <c r="AH199" s="10"/>
-      <c r="AK199" s="12"/>
+      <c r="AK199" s="16"/>
     </row>
     <row r="200" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D200" s="1"/>
@@ -3010,7 +3003,7 @@
       <c r="AA200" s="2"/>
       <c r="AG200" s="11"/>
       <c r="AH200" s="10"/>
-      <c r="AK200" s="12"/>
+      <c r="AK200" s="16"/>
     </row>
     <row r="201" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D201" s="1"/>
@@ -3021,7 +3014,7 @@
       <c r="AA201" s="2"/>
       <c r="AG201" s="11"/>
       <c r="AH201" s="10"/>
-      <c r="AK201" s="12"/>
+      <c r="AK201" s="16"/>
     </row>
     <row r="202" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D202" s="1"/>
@@ -3032,7 +3025,7 @@
       <c r="AA202" s="2"/>
       <c r="AG202" s="11"/>
       <c r="AH202" s="10"/>
-      <c r="AK202" s="12"/>
+      <c r="AK202" s="16"/>
     </row>
     <row r="203" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D203" s="1"/>
@@ -3043,7 +3036,7 @@
       <c r="AA203" s="2"/>
       <c r="AG203" s="11"/>
       <c r="AH203" s="10"/>
-      <c r="AK203" s="12"/>
+      <c r="AK203" s="16"/>
     </row>
     <row r="204" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D204" s="1"/>
@@ -3054,7 +3047,7 @@
       <c r="AA204" s="2"/>
       <c r="AG204" s="11"/>
       <c r="AH204" s="10"/>
-      <c r="AK204" s="12"/>
+      <c r="AK204" s="16"/>
     </row>
     <row r="205" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D205" s="1"/>
@@ -3065,7 +3058,7 @@
       <c r="AA205" s="2"/>
       <c r="AG205" s="11"/>
       <c r="AH205" s="10"/>
-      <c r="AK205" s="12"/>
+      <c r="AK205" s="16"/>
     </row>
     <row r="206" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D206" s="1"/>
@@ -3076,7 +3069,7 @@
       <c r="AA206" s="2"/>
       <c r="AG206" s="11"/>
       <c r="AH206" s="10"/>
-      <c r="AK206" s="12"/>
+      <c r="AK206" s="16"/>
     </row>
     <row r="207" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D207" s="1"/>
@@ -3087,7 +3080,7 @@
       <c r="AA207" s="2"/>
       <c r="AG207" s="11"/>
       <c r="AH207" s="10"/>
-      <c r="AK207" s="12"/>
+      <c r="AK207" s="16"/>
     </row>
     <row r="208" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D208" s="1"/>
@@ -3098,7 +3091,7 @@
       <c r="AA208" s="2"/>
       <c r="AG208" s="11"/>
       <c r="AH208" s="10"/>
-      <c r="AK208" s="12"/>
+      <c r="AK208" s="16"/>
     </row>
     <row r="209" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D209" s="1"/>
@@ -3109,7 +3102,7 @@
       <c r="AA209" s="2"/>
       <c r="AG209" s="11"/>
       <c r="AH209" s="10"/>
-      <c r="AK209" s="12"/>
+      <c r="AK209" s="16"/>
     </row>
     <row r="210" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D210" s="1"/>
@@ -3120,7 +3113,7 @@
       <c r="AA210" s="2"/>
       <c r="AG210" s="11"/>
       <c r="AH210" s="10"/>
-      <c r="AK210" s="12"/>
+      <c r="AK210" s="16"/>
     </row>
     <row r="211" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D211" s="1"/>
@@ -3131,7 +3124,7 @@
       <c r="AA211" s="2"/>
       <c r="AG211" s="11"/>
       <c r="AH211" s="10"/>
-      <c r="AK211" s="12"/>
+      <c r="AK211" s="16"/>
     </row>
     <row r="212" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D212" s="1"/>
@@ -3142,7 +3135,7 @@
       <c r="AA212" s="2"/>
       <c r="AG212" s="11"/>
       <c r="AH212" s="10"/>
-      <c r="AK212" s="12"/>
+      <c r="AK212" s="16"/>
     </row>
     <row r="213" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D213" s="1"/>
@@ -3153,7 +3146,7 @@
       <c r="AA213" s="2"/>
       <c r="AG213" s="11"/>
       <c r="AH213" s="10"/>
-      <c r="AK213" s="12"/>
+      <c r="AK213" s="16"/>
     </row>
     <row r="214" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D214" s="1"/>
@@ -3164,7 +3157,7 @@
       <c r="AA214" s="2"/>
       <c r="AG214" s="11"/>
       <c r="AH214" s="10"/>
-      <c r="AK214" s="12"/>
+      <c r="AK214" s="16"/>
     </row>
     <row r="215" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D215" s="1"/>
@@ -3175,7 +3168,7 @@
       <c r="AA215" s="2"/>
       <c r="AG215" s="11"/>
       <c r="AH215" s="10"/>
-      <c r="AK215" s="12"/>
+      <c r="AK215" s="16"/>
     </row>
     <row r="216" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D216" s="1"/>
@@ -3186,7 +3179,7 @@
       <c r="AA216" s="2"/>
       <c r="AG216" s="11"/>
       <c r="AH216" s="10"/>
-      <c r="AK216" s="12"/>
+      <c r="AK216" s="16"/>
     </row>
     <row r="217" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D217" s="1"/>
@@ -3197,7 +3190,7 @@
       <c r="AA217" s="2"/>
       <c r="AG217" s="11"/>
       <c r="AH217" s="10"/>
-      <c r="AK217" s="12"/>
+      <c r="AK217" s="16"/>
     </row>
     <row r="218" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D218" s="1"/>
@@ -3208,7 +3201,7 @@
       <c r="AA218" s="2"/>
       <c r="AG218" s="11"/>
       <c r="AH218" s="10"/>
-      <c r="AK218" s="12"/>
+      <c r="AK218" s="16"/>
     </row>
     <row r="219" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D219" s="1"/>
@@ -3219,7 +3212,7 @@
       <c r="AA219" s="2"/>
       <c r="AG219" s="11"/>
       <c r="AH219" s="10"/>
-      <c r="AK219" s="12"/>
+      <c r="AK219" s="16"/>
     </row>
     <row r="220" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D220" s="1"/>
@@ -3230,7 +3223,7 @@
       <c r="AA220" s="2"/>
       <c r="AG220" s="11"/>
       <c r="AH220" s="10"/>
-      <c r="AK220" s="12"/>
+      <c r="AK220" s="16"/>
     </row>
     <row r="221" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D221" s="1"/>
@@ -3241,7 +3234,7 @@
       <c r="AA221" s="2"/>
       <c r="AG221" s="11"/>
       <c r="AH221" s="10"/>
-      <c r="AK221" s="12"/>
+      <c r="AK221" s="16"/>
     </row>
     <row r="222" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D222" s="1"/>
@@ -3252,7 +3245,7 @@
       <c r="AA222" s="2"/>
       <c r="AG222" s="11"/>
       <c r="AH222" s="10"/>
-      <c r="AK222" s="12"/>
+      <c r="AK222" s="16"/>
     </row>
     <row r="223" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D223" s="1"/>
@@ -3263,7 +3256,7 @@
       <c r="AA223" s="2"/>
       <c r="AG223" s="11"/>
       <c r="AH223" s="10"/>
-      <c r="AK223" s="12"/>
+      <c r="AK223" s="16"/>
     </row>
     <row r="224" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D224" s="1"/>
@@ -3274,7 +3267,7 @@
       <c r="AA224" s="2"/>
       <c r="AG224" s="11"/>
       <c r="AH224" s="10"/>
-      <c r="AK224" s="12"/>
+      <c r="AK224" s="16"/>
     </row>
     <row r="225" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D225" s="1"/>
@@ -3285,7 +3278,7 @@
       <c r="AA225" s="2"/>
       <c r="AG225" s="11"/>
       <c r="AH225" s="10"/>
-      <c r="AK225" s="12"/>
+      <c r="AK225" s="16"/>
     </row>
     <row r="226" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D226" s="1"/>
@@ -3296,7 +3289,7 @@
       <c r="AA226" s="2"/>
       <c r="AG226" s="11"/>
       <c r="AH226" s="10"/>
-      <c r="AK226" s="12"/>
+      <c r="AK226" s="16"/>
     </row>
     <row r="227" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D227" s="1"/>
@@ -3307,7 +3300,7 @@
       <c r="AA227" s="2"/>
       <c r="AG227" s="11"/>
       <c r="AH227" s="10"/>
-      <c r="AK227" s="12"/>
+      <c r="AK227" s="16"/>
     </row>
     <row r="228" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D228" s="1"/>
@@ -3318,7 +3311,7 @@
       <c r="AA228" s="2"/>
       <c r="AG228" s="11"/>
       <c r="AH228" s="10"/>
-      <c r="AK228" s="12"/>
+      <c r="AK228" s="16"/>
     </row>
     <row r="229" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D229" s="1"/>
@@ -3329,7 +3322,7 @@
       <c r="AA229" s="2"/>
       <c r="AG229" s="11"/>
       <c r="AH229" s="10"/>
-      <c r="AK229" s="12"/>
+      <c r="AK229" s="16"/>
     </row>
     <row r="230" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D230" s="1"/>
@@ -3340,7 +3333,7 @@
       <c r="AA230" s="2"/>
       <c r="AG230" s="11"/>
       <c r="AH230" s="10"/>
-      <c r="AK230" s="12"/>
+      <c r="AK230" s="16"/>
     </row>
     <row r="231" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D231" s="1"/>
@@ -3351,7 +3344,7 @@
       <c r="AA231" s="2"/>
       <c r="AG231" s="11"/>
       <c r="AH231" s="10"/>
-      <c r="AK231" s="12"/>
+      <c r="AK231" s="16"/>
     </row>
     <row r="232" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D232" s="1"/>
@@ -3362,7 +3355,7 @@
       <c r="AA232" s="2"/>
       <c r="AG232" s="11"/>
       <c r="AH232" s="10"/>
-      <c r="AK232" s="12"/>
+      <c r="AK232" s="16"/>
     </row>
     <row r="233" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D233" s="1"/>
@@ -3373,7 +3366,7 @@
       <c r="AA233" s="2"/>
       <c r="AG233" s="11"/>
       <c r="AH233" s="10"/>
-      <c r="AK233" s="12"/>
+      <c r="AK233" s="16"/>
     </row>
     <row r="234" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D234" s="1"/>
@@ -3384,7 +3377,7 @@
       <c r="AA234" s="2"/>
       <c r="AG234" s="11"/>
       <c r="AH234" s="10"/>
-      <c r="AK234" s="12"/>
+      <c r="AK234" s="16"/>
     </row>
     <row r="235" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D235" s="1"/>
@@ -3395,7 +3388,7 @@
       <c r="AA235" s="2"/>
       <c r="AG235" s="11"/>
       <c r="AH235" s="10"/>
-      <c r="AK235" s="12"/>
+      <c r="AK235" s="16"/>
     </row>
     <row r="236" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D236" s="1"/>
@@ -3406,7 +3399,7 @@
       <c r="AA236" s="2"/>
       <c r="AG236" s="11"/>
       <c r="AH236" s="10"/>
-      <c r="AK236" s="12"/>
+      <c r="AK236" s="16"/>
     </row>
     <row r="237" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D237" s="1"/>
@@ -3417,7 +3410,7 @@
       <c r="AA237" s="2"/>
       <c r="AG237" s="11"/>
       <c r="AH237" s="10"/>
-      <c r="AK237" s="12"/>
+      <c r="AK237" s="16"/>
     </row>
     <row r="238" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D238" s="1"/>
@@ -3428,7 +3421,7 @@
       <c r="AA238" s="2"/>
       <c r="AG238" s="11"/>
       <c r="AH238" s="10"/>
-      <c r="AK238" s="12"/>
+      <c r="AK238" s="16"/>
     </row>
     <row r="239" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D239" s="1"/>
@@ -3439,7 +3432,7 @@
       <c r="AA239" s="2"/>
       <c r="AG239" s="11"/>
       <c r="AH239" s="10"/>
-      <c r="AK239" s="12"/>
+      <c r="AK239" s="16"/>
     </row>
     <row r="240" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D240" s="1"/>
@@ -3450,7 +3443,7 @@
       <c r="AA240" s="2"/>
       <c r="AG240" s="11"/>
       <c r="AH240" s="10"/>
-      <c r="AK240" s="12"/>
+      <c r="AK240" s="16"/>
     </row>
     <row r="241" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D241" s="1"/>
@@ -3461,7 +3454,7 @@
       <c r="AA241" s="2"/>
       <c r="AG241" s="11"/>
       <c r="AH241" s="10"/>
-      <c r="AK241" s="12"/>
+      <c r="AK241" s="16"/>
     </row>
     <row r="242" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D242" s="1"/>
@@ -3472,7 +3465,7 @@
       <c r="AA242" s="2"/>
       <c r="AG242" s="11"/>
       <c r="AH242" s="10"/>
-      <c r="AK242" s="12"/>
+      <c r="AK242" s="16"/>
     </row>
     <row r="243" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D243" s="1"/>
@@ -3483,7 +3476,7 @@
       <c r="AA243" s="2"/>
       <c r="AG243" s="11"/>
       <c r="AH243" s="10"/>
-      <c r="AK243" s="12"/>
+      <c r="AK243" s="16"/>
     </row>
     <row r="244" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D244" s="1"/>
@@ -3494,7 +3487,7 @@
       <c r="AA244" s="2"/>
       <c r="AG244" s="11"/>
       <c r="AH244" s="10"/>
-      <c r="AK244" s="12"/>
+      <c r="AK244" s="16"/>
     </row>
     <row r="245" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D245" s="1"/>
@@ -3505,7 +3498,7 @@
       <c r="AA245" s="2"/>
       <c r="AG245" s="11"/>
       <c r="AH245" s="10"/>
-      <c r="AK245" s="12"/>
+      <c r="AK245" s="16"/>
     </row>
     <row r="246" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D246" s="1"/>
@@ -3516,7 +3509,7 @@
       <c r="AA246" s="2"/>
       <c r="AG246" s="11"/>
       <c r="AH246" s="10"/>
-      <c r="AK246" s="12"/>
+      <c r="AK246" s="16"/>
     </row>
     <row r="247" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D247" s="1"/>
@@ -3527,7 +3520,7 @@
       <c r="AA247" s="2"/>
       <c r="AG247" s="11"/>
       <c r="AH247" s="10"/>
-      <c r="AK247" s="12"/>
+      <c r="AK247" s="16"/>
     </row>
     <row r="248" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D248" s="1"/>
@@ -3538,7 +3531,7 @@
       <c r="AA248" s="2"/>
       <c r="AG248" s="11"/>
       <c r="AH248" s="10"/>
-      <c r="AK248" s="12"/>
+      <c r="AK248" s="16"/>
     </row>
     <row r="249" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D249" s="1"/>
@@ -3549,7 +3542,7 @@
       <c r="AA249" s="2"/>
       <c r="AG249" s="11"/>
       <c r="AH249" s="10"/>
-      <c r="AK249" s="12"/>
+      <c r="AK249" s="16"/>
     </row>
     <row r="250" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D250" s="1"/>
@@ -3560,7 +3553,7 @@
       <c r="AA250" s="2"/>
       <c r="AG250" s="11"/>
       <c r="AH250" s="10"/>
-      <c r="AK250" s="12"/>
+      <c r="AK250" s="16"/>
     </row>
     <row r="251" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D251" s="1"/>
@@ -3571,7 +3564,7 @@
       <c r="AA251" s="2"/>
       <c r="AG251" s="11"/>
       <c r="AH251" s="10"/>
-      <c r="AK251" s="12"/>
+      <c r="AK251" s="16"/>
     </row>
     <row r="252" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D252" s="1"/>
@@ -3582,7 +3575,7 @@
       <c r="AA252" s="2"/>
       <c r="AG252" s="11"/>
       <c r="AH252" s="10"/>
-      <c r="AK252" s="12"/>
+      <c r="AK252" s="16"/>
     </row>
     <row r="253" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D253" s="1"/>
@@ -3593,7 +3586,7 @@
       <c r="AA253" s="2"/>
       <c r="AG253" s="11"/>
       <c r="AH253" s="10"/>
-      <c r="AK253" s="12"/>
+      <c r="AK253" s="16"/>
     </row>
     <row r="254" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D254" s="1"/>
@@ -3604,7 +3597,7 @@
       <c r="AA254" s="2"/>
       <c r="AG254" s="11"/>
       <c r="AH254" s="10"/>
-      <c r="AK254" s="12"/>
+      <c r="AK254" s="16"/>
     </row>
     <row r="255" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D255" s="1"/>
@@ -3615,7 +3608,7 @@
       <c r="AA255" s="2"/>
       <c r="AG255" s="11"/>
       <c r="AH255" s="10"/>
-      <c r="AK255" s="12"/>
+      <c r="AK255" s="16"/>
     </row>
     <row r="256" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D256" s="1"/>
@@ -3626,7 +3619,7 @@
       <c r="AA256" s="2"/>
       <c r="AG256" s="11"/>
       <c r="AH256" s="10"/>
-      <c r="AK256" s="12"/>
+      <c r="AK256" s="16"/>
     </row>
     <row r="257" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D257" s="1"/>
@@ -3637,7 +3630,7 @@
       <c r="AA257" s="2"/>
       <c r="AG257" s="11"/>
       <c r="AH257" s="10"/>
-      <c r="AK257" s="12"/>
+      <c r="AK257" s="16"/>
     </row>
     <row r="258" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D258" s="1"/>
@@ -3648,7 +3641,7 @@
       <c r="AA258" s="2"/>
       <c r="AG258" s="11"/>
       <c r="AH258" s="10"/>
-      <c r="AK258" s="12"/>
+      <c r="AK258" s="16"/>
     </row>
     <row r="259" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D259" s="1"/>
@@ -3659,7 +3652,7 @@
       <c r="AA259" s="2"/>
       <c r="AG259" s="11"/>
       <c r="AH259" s="10"/>
-      <c r="AK259" s="12"/>
+      <c r="AK259" s="16"/>
     </row>
     <row r="260" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D260" s="1"/>
@@ -3670,7 +3663,7 @@
       <c r="AA260" s="2"/>
       <c r="AG260" s="11"/>
       <c r="AH260" s="10"/>
-      <c r="AK260" s="12"/>
+      <c r="AK260" s="16"/>
     </row>
     <row r="261" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D261" s="1"/>
@@ -3681,7 +3674,7 @@
       <c r="AA261" s="2"/>
       <c r="AG261" s="11"/>
       <c r="AH261" s="10"/>
-      <c r="AK261" s="12"/>
+      <c r="AK261" s="16"/>
     </row>
     <row r="262" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D262" s="1"/>
@@ -3692,7 +3685,7 @@
       <c r="AA262" s="2"/>
       <c r="AG262" s="11"/>
       <c r="AH262" s="10"/>
-      <c r="AK262" s="12"/>
+      <c r="AK262" s="16"/>
     </row>
     <row r="263" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D263" s="1"/>
@@ -3703,7 +3696,7 @@
       <c r="AA263" s="2"/>
       <c r="AG263" s="11"/>
       <c r="AH263" s="10"/>
-      <c r="AK263" s="12"/>
+      <c r="AK263" s="16"/>
     </row>
     <row r="264" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D264" s="1"/>
@@ -3714,7 +3707,7 @@
       <c r="AA264" s="2"/>
       <c r="AG264" s="11"/>
       <c r="AH264" s="10"/>
-      <c r="AK264" s="12"/>
+      <c r="AK264" s="16"/>
     </row>
     <row r="265" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D265" s="1"/>
@@ -3725,7 +3718,7 @@
       <c r="AA265" s="2"/>
       <c r="AG265" s="11"/>
       <c r="AH265" s="10"/>
-      <c r="AK265" s="12"/>
+      <c r="AK265" s="16"/>
     </row>
     <row r="266" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D266" s="1"/>
@@ -3736,7 +3729,7 @@
       <c r="AA266" s="2"/>
       <c r="AG266" s="11"/>
       <c r="AH266" s="10"/>
-      <c r="AK266" s="12"/>
+      <c r="AK266" s="16"/>
     </row>
     <row r="267" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D267" s="1"/>
@@ -3747,7 +3740,7 @@
       <c r="AA267" s="2"/>
       <c r="AG267" s="11"/>
       <c r="AH267" s="10"/>
-      <c r="AK267" s="12"/>
+      <c r="AK267" s="16"/>
     </row>
     <row r="268" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D268" s="1"/>
@@ -3758,7 +3751,7 @@
       <c r="AA268" s="2"/>
       <c r="AG268" s="11"/>
       <c r="AH268" s="10"/>
-      <c r="AK268" s="12"/>
+      <c r="AK268" s="16"/>
     </row>
     <row r="269" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D269" s="1"/>
@@ -3769,7 +3762,7 @@
       <c r="AA269" s="2"/>
       <c r="AG269" s="11"/>
       <c r="AH269" s="10"/>
-      <c r="AK269" s="12"/>
+      <c r="AK269" s="16"/>
     </row>
     <row r="270" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D270" s="1"/>
@@ -3780,7 +3773,7 @@
       <c r="AA270" s="2"/>
       <c r="AG270" s="11"/>
       <c r="AH270" s="10"/>
-      <c r="AK270" s="12"/>
+      <c r="AK270" s="16"/>
     </row>
     <row r="271" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D271" s="1"/>
@@ -3791,7 +3784,7 @@
       <c r="AA271" s="2"/>
       <c r="AG271" s="11"/>
       <c r="AH271" s="10"/>
-      <c r="AK271" s="12"/>
+      <c r="AK271" s="16"/>
     </row>
     <row r="272" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D272" s="1"/>
@@ -3802,7 +3795,7 @@
       <c r="AA272" s="2"/>
       <c r="AG272" s="11"/>
       <c r="AH272" s="10"/>
-      <c r="AK272" s="12"/>
+      <c r="AK272" s="16"/>
     </row>
     <row r="273" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D273" s="1"/>
@@ -3813,7 +3806,7 @@
       <c r="AA273" s="2"/>
       <c r="AG273" s="11"/>
       <c r="AH273" s="10"/>
-      <c r="AK273" s="12"/>
+      <c r="AK273" s="16"/>
     </row>
     <row r="274" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D274" s="1"/>
@@ -3824,7 +3817,7 @@
       <c r="AA274" s="2"/>
       <c r="AG274" s="11"/>
       <c r="AH274" s="10"/>
-      <c r="AK274" s="12"/>
+      <c r="AK274" s="16"/>
     </row>
     <row r="275" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D275" s="1"/>
@@ -3835,7 +3828,7 @@
       <c r="AA275" s="2"/>
       <c r="AG275" s="11"/>
       <c r="AH275" s="10"/>
-      <c r="AK275" s="12"/>
+      <c r="AK275" s="16"/>
     </row>
     <row r="276" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D276" s="1"/>
@@ -3846,7 +3839,7 @@
       <c r="AA276" s="2"/>
       <c r="AG276" s="11"/>
       <c r="AH276" s="10"/>
-      <c r="AK276" s="12"/>
+      <c r="AK276" s="16"/>
     </row>
     <row r="277" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D277" s="1"/>
@@ -3857,7 +3850,7 @@
       <c r="AA277" s="2"/>
       <c r="AG277" s="11"/>
       <c r="AH277" s="10"/>
-      <c r="AK277" s="12"/>
+      <c r="AK277" s="16"/>
     </row>
     <row r="278" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D278" s="1"/>
@@ -3868,7 +3861,7 @@
       <c r="AA278" s="2"/>
       <c r="AG278" s="11"/>
       <c r="AH278" s="10"/>
-      <c r="AK278" s="12"/>
+      <c r="AK278" s="16"/>
     </row>
     <row r="279" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D279" s="1"/>
@@ -3879,7 +3872,7 @@
       <c r="AA279" s="2"/>
       <c r="AG279" s="11"/>
       <c r="AH279" s="10"/>
-      <c r="AK279" s="12"/>
+      <c r="AK279" s="16"/>
     </row>
     <row r="280" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D280" s="1"/>
@@ -3890,7 +3883,7 @@
       <c r="AA280" s="2"/>
       <c r="AG280" s="11"/>
       <c r="AH280" s="10"/>
-      <c r="AK280" s="12"/>
+      <c r="AK280" s="16"/>
     </row>
     <row r="281" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D281" s="1"/>
@@ -3901,7 +3894,7 @@
       <c r="AA281" s="2"/>
       <c r="AG281" s="11"/>
       <c r="AH281" s="10"/>
-      <c r="AK281" s="12"/>
+      <c r="AK281" s="16"/>
     </row>
     <row r="282" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D282" s="1"/>
@@ -3912,7 +3905,7 @@
       <c r="AA282" s="2"/>
       <c r="AG282" s="11"/>
       <c r="AH282" s="10"/>
-      <c r="AK282" s="12"/>
+      <c r="AK282" s="16"/>
     </row>
     <row r="283" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D283" s="1"/>
@@ -3923,7 +3916,7 @@
       <c r="AA283" s="2"/>
       <c r="AG283" s="11"/>
       <c r="AH283" s="10"/>
-      <c r="AK283" s="12"/>
+      <c r="AK283" s="16"/>
     </row>
     <row r="284" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D284" s="1"/>
@@ -3934,7 +3927,7 @@
       <c r="AA284" s="2"/>
       <c r="AG284" s="11"/>
       <c r="AH284" s="10"/>
-      <c r="AK284" s="12"/>
+      <c r="AK284" s="16"/>
     </row>
     <row r="285" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D285" s="1"/>
@@ -3945,7 +3938,7 @@
       <c r="AA285" s="2"/>
       <c r="AG285" s="11"/>
       <c r="AH285" s="10"/>
-      <c r="AK285" s="12"/>
+      <c r="AK285" s="16"/>
     </row>
     <row r="286" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D286" s="1"/>
@@ -3956,7 +3949,7 @@
       <c r="AA286" s="2"/>
       <c r="AG286" s="11"/>
       <c r="AH286" s="10"/>
-      <c r="AK286" s="12"/>
+      <c r="AK286" s="16"/>
     </row>
     <row r="287" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D287" s="1"/>
@@ -3967,7 +3960,7 @@
       <c r="AA287" s="2"/>
       <c r="AG287" s="11"/>
       <c r="AH287" s="10"/>
-      <c r="AK287" s="12"/>
+      <c r="AK287" s="16"/>
     </row>
     <row r="288" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D288" s="1"/>
@@ -3978,7 +3971,7 @@
       <c r="AA288" s="2"/>
       <c r="AG288" s="11"/>
       <c r="AH288" s="10"/>
-      <c r="AK288" s="12"/>
+      <c r="AK288" s="16"/>
     </row>
     <row r="289" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D289" s="1"/>
@@ -3989,7 +3982,7 @@
       <c r="AA289" s="2"/>
       <c r="AG289" s="11"/>
       <c r="AH289" s="10"/>
-      <c r="AK289" s="12"/>
+      <c r="AK289" s="16"/>
     </row>
     <row r="290" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D290" s="1"/>
@@ -4000,7 +3993,7 @@
       <c r="AA290" s="2"/>
       <c r="AG290" s="11"/>
       <c r="AH290" s="10"/>
-      <c r="AK290" s="12"/>
+      <c r="AK290" s="16"/>
     </row>
     <row r="291" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D291" s="1"/>
@@ -4011,7 +4004,7 @@
       <c r="AA291" s="2"/>
       <c r="AG291" s="11"/>
       <c r="AH291" s="10"/>
-      <c r="AK291" s="12"/>
+      <c r="AK291" s="16"/>
     </row>
     <row r="292" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D292" s="1"/>
@@ -4022,7 +4015,7 @@
       <c r="AA292" s="2"/>
       <c r="AG292" s="11"/>
       <c r="AH292" s="10"/>
-      <c r="AK292" s="12"/>
+      <c r="AK292" s="16"/>
     </row>
     <row r="293" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D293" s="1"/>
@@ -4033,7 +4026,7 @@
       <c r="AA293" s="2"/>
       <c r="AG293" s="11"/>
       <c r="AH293" s="10"/>
-      <c r="AK293" s="12"/>
+      <c r="AK293" s="16"/>
     </row>
     <row r="294" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D294" s="1"/>
@@ -4044,7 +4037,7 @@
       <c r="AA294" s="2"/>
       <c r="AG294" s="11"/>
       <c r="AH294" s="10"/>
-      <c r="AK294" s="12"/>
+      <c r="AK294" s="16"/>
     </row>
     <row r="295" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D295" s="1"/>
@@ -4055,7 +4048,7 @@
       <c r="AA295" s="2"/>
       <c r="AG295" s="11"/>
       <c r="AH295" s="10"/>
-      <c r="AK295" s="12"/>
+      <c r="AK295" s="16"/>
     </row>
     <row r="296" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D296" s="1"/>
@@ -4066,7 +4059,7 @@
       <c r="AA296" s="2"/>
       <c r="AG296" s="11"/>
       <c r="AH296" s="10"/>
-      <c r="AK296" s="12"/>
+      <c r="AK296" s="16"/>
     </row>
     <row r="297" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D297" s="1"/>
@@ -4077,7 +4070,7 @@
       <c r="AA297" s="2"/>
       <c r="AG297" s="11"/>
       <c r="AH297" s="10"/>
-      <c r="AK297" s="12"/>
+      <c r="AK297" s="16"/>
     </row>
     <row r="298" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D298" s="1"/>
@@ -4088,7 +4081,7 @@
       <c r="AA298" s="2"/>
       <c r="AG298" s="11"/>
       <c r="AH298" s="10"/>
-      <c r="AK298" s="12"/>
+      <c r="AK298" s="16"/>
     </row>
     <row r="299" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D299" s="1"/>
@@ -4099,7 +4092,7 @@
       <c r="AA299" s="2"/>
       <c r="AG299" s="11"/>
       <c r="AH299" s="10"/>
-      <c r="AK299" s="12"/>
+      <c r="AK299" s="16"/>
     </row>
     <row r="300" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D300" s="1"/>
@@ -4110,7 +4103,7 @@
       <c r="AA300" s="2"/>
       <c r="AG300" s="11"/>
       <c r="AH300" s="10"/>
-      <c r="AK300" s="12"/>
+      <c r="AK300" s="16"/>
     </row>
     <row r="301" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D301" s="1"/>
@@ -4121,7 +4114,7 @@
       <c r="AA301" s="2"/>
       <c r="AG301" s="11"/>
       <c r="AH301" s="10"/>
-      <c r="AK301" s="12"/>
+      <c r="AK301" s="16"/>
     </row>
     <row r="302" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D302" s="1"/>
@@ -4132,7 +4125,7 @@
       <c r="AA302" s="2"/>
       <c r="AG302" s="11"/>
       <c r="AH302" s="10"/>
-      <c r="AK302" s="12"/>
+      <c r="AK302" s="16"/>
     </row>
     <row r="303" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D303" s="1"/>
@@ -4143,7 +4136,7 @@
       <c r="AA303" s="2"/>
       <c r="AG303" s="11"/>
       <c r="AH303" s="10"/>
-      <c r="AK303" s="12"/>
+      <c r="AK303" s="16"/>
     </row>
     <row r="304" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D304" s="1"/>
@@ -4154,7 +4147,7 @@
       <c r="AA304" s="2"/>
       <c r="AG304" s="11"/>
       <c r="AH304" s="10"/>
-      <c r="AK304" s="12"/>
+      <c r="AK304" s="16"/>
     </row>
     <row r="305" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D305" s="1"/>
@@ -4165,7 +4158,7 @@
       <c r="AA305" s="2"/>
       <c r="AG305" s="11"/>
       <c r="AH305" s="10"/>
-      <c r="AK305" s="12"/>
+      <c r="AK305" s="16"/>
     </row>
     <row r="306" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D306" s="1"/>
@@ -4176,7 +4169,7 @@
       <c r="AA306" s="2"/>
       <c r="AG306" s="11"/>
       <c r="AH306" s="10"/>
-      <c r="AK306" s="12"/>
+      <c r="AK306" s="16"/>
     </row>
     <row r="307" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D307" s="1"/>
@@ -4187,7 +4180,7 @@
       <c r="AA307" s="2"/>
       <c r="AG307" s="11"/>
       <c r="AH307" s="10"/>
-      <c r="AK307" s="12"/>
+      <c r="AK307" s="16"/>
     </row>
     <row r="308" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D308" s="1"/>
@@ -4198,7 +4191,7 @@
       <c r="AA308" s="2"/>
       <c r="AG308" s="11"/>
       <c r="AH308" s="10"/>
-      <c r="AK308" s="12"/>
+      <c r="AK308" s="16"/>
     </row>
     <row r="309" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D309" s="1"/>
@@ -4209,7 +4202,7 @@
       <c r="AA309" s="2"/>
       <c r="AG309" s="11"/>
       <c r="AH309" s="10"/>
-      <c r="AK309" s="12"/>
+      <c r="AK309" s="16"/>
     </row>
     <row r="310" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D310" s="1"/>
@@ -4220,7 +4213,7 @@
       <c r="AA310" s="2"/>
       <c r="AG310" s="11"/>
       <c r="AH310" s="10"/>
-      <c r="AK310" s="12"/>
+      <c r="AK310" s="16"/>
     </row>
     <row r="311" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D311" s="1"/>
@@ -4231,7 +4224,7 @@
       <c r="AA311" s="2"/>
       <c r="AG311" s="11"/>
       <c r="AH311" s="10"/>
-      <c r="AK311" s="12"/>
+      <c r="AK311" s="16"/>
     </row>
     <row r="312" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D312" s="1"/>
@@ -4242,7 +4235,7 @@
       <c r="AA312" s="2"/>
       <c r="AG312" s="11"/>
       <c r="AH312" s="10"/>
-      <c r="AK312" s="12"/>
+      <c r="AK312" s="16"/>
     </row>
     <row r="313" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D313" s="1"/>
@@ -4253,7 +4246,7 @@
       <c r="AA313" s="2"/>
       <c r="AG313" s="11"/>
       <c r="AH313" s="10"/>
-      <c r="AK313" s="12"/>
+      <c r="AK313" s="16"/>
     </row>
     <row r="314" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D314" s="1"/>
@@ -4264,7 +4257,7 @@
       <c r="AA314" s="2"/>
       <c r="AG314" s="11"/>
       <c r="AH314" s="10"/>
-      <c r="AK314" s="12"/>
+      <c r="AK314" s="16"/>
     </row>
     <row r="315" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D315" s="1"/>
@@ -4275,7 +4268,7 @@
       <c r="AA315" s="2"/>
       <c r="AG315" s="11"/>
       <c r="AH315" s="10"/>
-      <c r="AK315" s="12"/>
+      <c r="AK315" s="16"/>
     </row>
     <row r="316" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D316" s="1"/>
@@ -4286,7 +4279,7 @@
       <c r="AA316" s="2"/>
       <c r="AG316" s="11"/>
       <c r="AH316" s="10"/>
-      <c r="AK316" s="12"/>
+      <c r="AK316" s="16"/>
     </row>
     <row r="317" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D317" s="1"/>
@@ -4297,7 +4290,7 @@
       <c r="AA317" s="2"/>
       <c r="AG317" s="11"/>
       <c r="AH317" s="10"/>
-      <c r="AK317" s="12"/>
+      <c r="AK317" s="16"/>
     </row>
     <row r="318" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D318" s="1"/>
@@ -4308,7 +4301,7 @@
       <c r="AA318" s="2"/>
       <c r="AG318" s="11"/>
       <c r="AH318" s="10"/>
-      <c r="AK318" s="12"/>
+      <c r="AK318" s="16"/>
     </row>
     <row r="319" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D319" s="1"/>
@@ -4319,7 +4312,7 @@
       <c r="AA319" s="2"/>
       <c r="AG319" s="11"/>
       <c r="AH319" s="10"/>
-      <c r="AK319" s="12"/>
+      <c r="AK319" s="16"/>
     </row>
     <row r="320" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D320" s="1"/>
@@ -4330,7 +4323,7 @@
       <c r="AA320" s="2"/>
       <c r="AG320" s="11"/>
       <c r="AH320" s="10"/>
-      <c r="AK320" s="12"/>
+      <c r="AK320" s="16"/>
     </row>
     <row r="321" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D321" s="1"/>
@@ -4341,7 +4334,7 @@
       <c r="AA321" s="2"/>
       <c r="AG321" s="11"/>
       <c r="AH321" s="10"/>
-      <c r="AK321" s="12"/>
+      <c r="AK321" s="16"/>
     </row>
     <row r="322" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D322" s="1"/>
@@ -4352,7 +4345,7 @@
       <c r="AA322" s="2"/>
       <c r="AG322" s="11"/>
       <c r="AH322" s="10"/>
-      <c r="AK322" s="12"/>
+      <c r="AK322" s="16"/>
     </row>
     <row r="323" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D323" s="1"/>
@@ -4363,7 +4356,7 @@
       <c r="AA323" s="2"/>
       <c r="AG323" s="11"/>
       <c r="AH323" s="10"/>
-      <c r="AK323" s="12"/>
+      <c r="AK323" s="16"/>
     </row>
     <row r="324" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D324" s="1"/>
@@ -4374,7 +4367,7 @@
       <c r="AA324" s="2"/>
       <c r="AG324" s="11"/>
       <c r="AH324" s="10"/>
-      <c r="AK324" s="12"/>
+      <c r="AK324" s="16"/>
     </row>
     <row r="325" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D325" s="1"/>
@@ -4385,7 +4378,7 @@
       <c r="AA325" s="2"/>
       <c r="AG325" s="11"/>
       <c r="AH325" s="10"/>
-      <c r="AK325" s="12"/>
+      <c r="AK325" s="16"/>
     </row>
     <row r="326" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D326" s="1"/>
@@ -4396,7 +4389,7 @@
       <c r="AA326" s="2"/>
       <c r="AG326" s="11"/>
       <c r="AH326" s="10"/>
-      <c r="AK326" s="12"/>
+      <c r="AK326" s="16"/>
     </row>
     <row r="327" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D327" s="1"/>
@@ -4407,7 +4400,7 @@
       <c r="AA327" s="2"/>
       <c r="AG327" s="11"/>
       <c r="AH327" s="10"/>
-      <c r="AK327" s="12"/>
+      <c r="AK327" s="16"/>
     </row>
     <row r="328" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D328" s="1"/>
@@ -4418,7 +4411,7 @@
       <c r="AA328" s="2"/>
       <c r="AG328" s="11"/>
       <c r="AH328" s="10"/>
-      <c r="AK328" s="12"/>
+      <c r="AK328" s="16"/>
     </row>
     <row r="329" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D329" s="1"/>
@@ -4429,7 +4422,7 @@
       <c r="AA329" s="2"/>
       <c r="AG329" s="11"/>
       <c r="AH329" s="10"/>
-      <c r="AK329" s="12"/>
+      <c r="AK329" s="16"/>
     </row>
     <row r="330" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D330" s="1"/>
@@ -4440,7 +4433,7 @@
       <c r="AA330" s="2"/>
       <c r="AG330" s="11"/>
       <c r="AH330" s="10"/>
-      <c r="AK330" s="12"/>
+      <c r="AK330" s="16"/>
     </row>
     <row r="331" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D331" s="1"/>
@@ -4451,7 +4444,7 @@
       <c r="AA331" s="2"/>
       <c r="AG331" s="11"/>
       <c r="AH331" s="10"/>
-      <c r="AK331" s="12"/>
+      <c r="AK331" s="16"/>
     </row>
     <row r="332" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D332" s="1"/>
@@ -4462,7 +4455,7 @@
       <c r="AA332" s="2"/>
       <c r="AG332" s="11"/>
       <c r="AH332" s="10"/>
-      <c r="AK332" s="12"/>
+      <c r="AK332" s="16"/>
     </row>
     <row r="333" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D333" s="1"/>
@@ -4473,7 +4466,7 @@
       <c r="AA333" s="2"/>
       <c r="AG333" s="11"/>
       <c r="AH333" s="10"/>
-      <c r="AK333" s="12"/>
+      <c r="AK333" s="16"/>
     </row>
     <row r="334" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D334" s="1"/>
@@ -4484,7 +4477,7 @@
       <c r="AA334" s="2"/>
       <c r="AG334" s="11"/>
       <c r="AH334" s="10"/>
-      <c r="AK334" s="12"/>
+      <c r="AK334" s="16"/>
     </row>
     <row r="335" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D335" s="1"/>
@@ -4495,7 +4488,7 @@
       <c r="AA335" s="2"/>
       <c r="AG335" s="11"/>
       <c r="AH335" s="10"/>
-      <c r="AK335" s="12"/>
+      <c r="AK335" s="16"/>
     </row>
     <row r="336" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D336" s="1"/>
@@ -4506,7 +4499,7 @@
       <c r="AA336" s="2"/>
       <c r="AG336" s="11"/>
       <c r="AH336" s="10"/>
-      <c r="AK336" s="12"/>
+      <c r="AK336" s="16"/>
     </row>
     <row r="337" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D337" s="1"/>
@@ -4517,7 +4510,7 @@
       <c r="AA337" s="2"/>
       <c r="AG337" s="11"/>
       <c r="AH337" s="10"/>
-      <c r="AK337" s="12"/>
+      <c r="AK337" s="16"/>
     </row>
     <row r="338" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D338" s="1"/>
@@ -4528,7 +4521,7 @@
       <c r="AA338" s="2"/>
       <c r="AG338" s="11"/>
       <c r="AH338" s="10"/>
-      <c r="AK338" s="12"/>
+      <c r="AK338" s="16"/>
     </row>
     <row r="339" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D339" s="1"/>
@@ -4539,7 +4532,7 @@
       <c r="AA339" s="2"/>
       <c r="AG339" s="11"/>
       <c r="AH339" s="10"/>
-      <c r="AK339" s="12"/>
+      <c r="AK339" s="16"/>
     </row>
     <row r="340" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D340" s="1"/>
@@ -4550,7 +4543,7 @@
       <c r="AA340" s="2"/>
       <c r="AG340" s="11"/>
       <c r="AH340" s="10"/>
-      <c r="AK340" s="12"/>
+      <c r="AK340" s="16"/>
     </row>
     <row r="341" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D341" s="1"/>
@@ -4561,7 +4554,7 @@
       <c r="AA341" s="2"/>
       <c r="AG341" s="11"/>
       <c r="AH341" s="10"/>
-      <c r="AK341" s="12"/>
+      <c r="AK341" s="16"/>
     </row>
     <row r="342" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D342" s="1"/>
@@ -4572,7 +4565,7 @@
       <c r="AA342" s="2"/>
       <c r="AG342" s="11"/>
       <c r="AH342" s="10"/>
-      <c r="AK342" s="12"/>
+      <c r="AK342" s="16"/>
     </row>
     <row r="343" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D343" s="1"/>
@@ -4583,7 +4576,7 @@
       <c r="AA343" s="2"/>
       <c r="AG343" s="11"/>
       <c r="AH343" s="10"/>
-      <c r="AK343" s="12"/>
+      <c r="AK343" s="16"/>
     </row>
     <row r="344" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D344" s="1"/>
@@ -4594,7 +4587,7 @@
       <c r="AA344" s="2"/>
       <c r="AG344" s="11"/>
       <c r="AH344" s="10"/>
-      <c r="AK344" s="12"/>
+      <c r="AK344" s="16"/>
     </row>
     <row r="345" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D345" s="1"/>
@@ -4605,7 +4598,7 @@
       <c r="AA345" s="2"/>
       <c r="AG345" s="11"/>
       <c r="AH345" s="10"/>
-      <c r="AK345" s="12"/>
+      <c r="AK345" s="16"/>
     </row>
     <row r="346" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D346" s="1"/>
@@ -4616,7 +4609,7 @@
       <c r="AA346" s="2"/>
       <c r="AG346" s="11"/>
       <c r="AH346" s="10"/>
-      <c r="AK346" s="12"/>
+      <c r="AK346" s="16"/>
     </row>
     <row r="347" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D347" s="1"/>
@@ -4627,7 +4620,7 @@
       <c r="AA347" s="2"/>
       <c r="AG347" s="11"/>
       <c r="AH347" s="10"/>
-      <c r="AK347" s="12"/>
+      <c r="AK347" s="16"/>
     </row>
     <row r="348" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D348" s="1"/>
@@ -4638,7 +4631,7 @@
       <c r="AA348" s="2"/>
       <c r="AG348" s="11"/>
       <c r="AH348" s="10"/>
-      <c r="AK348" s="12"/>
+      <c r="AK348" s="16"/>
     </row>
     <row r="349" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D349" s="1"/>
@@ -4649,7 +4642,7 @@
       <c r="AA349" s="2"/>
       <c r="AG349" s="11"/>
       <c r="AH349" s="10"/>
-      <c r="AK349" s="12"/>
+      <c r="AK349" s="16"/>
     </row>
     <row r="350" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D350" s="1"/>
@@ -4660,7 +4653,7 @@
       <c r="AA350" s="2"/>
       <c r="AG350" s="11"/>
       <c r="AH350" s="10"/>
-      <c r="AK350" s="12"/>
+      <c r="AK350" s="16"/>
     </row>
     <row r="351" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D351" s="1"/>
@@ -4671,7 +4664,7 @@
       <c r="AA351" s="2"/>
       <c r="AG351" s="11"/>
       <c r="AH351" s="10"/>
-      <c r="AK351" s="12"/>
+      <c r="AK351" s="16"/>
     </row>
     <row r="352" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D352" s="1"/>
@@ -4682,7 +4675,7 @@
       <c r="AA352" s="2"/>
       <c r="AG352" s="11"/>
       <c r="AH352" s="10"/>
-      <c r="AK352" s="12"/>
+      <c r="AK352" s="16"/>
     </row>
     <row r="353" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D353" s="1"/>
@@ -4693,7 +4686,7 @@
       <c r="AA353" s="2"/>
       <c r="AG353" s="11"/>
       <c r="AH353" s="10"/>
-      <c r="AK353" s="12"/>
+      <c r="AK353" s="16"/>
     </row>
     <row r="354" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D354" s="1"/>
@@ -4704,7 +4697,7 @@
       <c r="AA354" s="2"/>
       <c r="AG354" s="11"/>
       <c r="AH354" s="10"/>
-      <c r="AK354" s="12"/>
+      <c r="AK354" s="16"/>
     </row>
     <row r="355" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D355" s="1"/>
@@ -4715,7 +4708,7 @@
       <c r="AA355" s="2"/>
       <c r="AG355" s="11"/>
       <c r="AH355" s="10"/>
-      <c r="AK355" s="12"/>
+      <c r="AK355" s="16"/>
     </row>
     <row r="356" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D356" s="1"/>
@@ -4726,7 +4719,7 @@
       <c r="AA356" s="2"/>
       <c r="AG356" s="11"/>
       <c r="AH356" s="10"/>
-      <c r="AK356" s="12"/>
+      <c r="AK356" s="16"/>
     </row>
     <row r="357" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D357" s="1"/>
@@ -4737,7 +4730,7 @@
       <c r="AA357" s="2"/>
       <c r="AG357" s="11"/>
       <c r="AH357" s="10"/>
-      <c r="AK357" s="12"/>
+      <c r="AK357" s="16"/>
     </row>
     <row r="358" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D358" s="1"/>
@@ -4748,7 +4741,7 @@
       <c r="AA358" s="2"/>
       <c r="AG358" s="11"/>
       <c r="AH358" s="10"/>
-      <c r="AK358" s="12"/>
+      <c r="AK358" s="16"/>
     </row>
     <row r="359" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D359" s="1"/>
@@ -4759,7 +4752,7 @@
       <c r="AA359" s="2"/>
       <c r="AG359" s="11"/>
       <c r="AH359" s="10"/>
-      <c r="AK359" s="12"/>
+      <c r="AK359" s="16"/>
     </row>
     <row r="360" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D360" s="1"/>
@@ -4770,7 +4763,7 @@
       <c r="AA360" s="2"/>
       <c r="AG360" s="11"/>
       <c r="AH360" s="10"/>
-      <c r="AK360" s="12"/>
+      <c r="AK360" s="16"/>
     </row>
     <row r="361" spans="4:37" x14ac:dyDescent="0.35">
       <c r="D361" s="1"/>
@@ -4781,7 +4774,7 @@
       <c r="AA361" s="2"/>
       <c r="AG361" s="11"/>
       <c r="AH361" s="10"/>
-      <c r="AK361" s="12"/>
+      <c r="AK361" s="16"/>
     </row>
   </sheetData>
   <protectedRanges>

</xml_diff>